<commit_message>
chg ! write error messages into imported excel file
</commit_message>
<xml_diff>
--- a/tests/data/rdi_one.xlsx
+++ b/tests/data/rdi_one.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Households" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,7 +13,7 @@
     <sheet name="People" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Individuals!$A$1:$R$369</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Individuals!$B$1:$S$354</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="108">
   <si>
     <t xml:space="preserve">household_id</t>
   </si>
@@ -72,6 +72,9 @@
     <t xml:space="preserve">first_registration_date_h_c</t>
   </si>
   <si>
+    <t xml:space="preserve">head_of_household_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">MDG</t>
   </si>
   <si>
@@ -91,6 +94,9 @@
   </si>
   <si>
     <t xml:space="preserve">unicef government_partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">individual_id</t>
   </si>
   <si>
     <t xml:space="preserve">relationship_i_c</t>
@@ -540,16 +546,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>70</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>727560</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>108720</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>726840</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>108000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -562,8 +568,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16229160" y="13335120"/>
-          <a:ext cx="727560" cy="299160"/>
+          <a:off x="17254800" y="10477440"/>
+          <a:ext cx="726840" cy="298440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -577,16 +583,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>96840</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>96120</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>93240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -599,8 +605,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9654480" y="762120"/>
-          <a:ext cx="96840" cy="93960"/>
+          <a:off x="10680120" y="762120"/>
+          <a:ext cx="96120" cy="93240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -626,9 +632,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>96840</xdr:colOff>
+      <xdr:colOff>96120</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -642,7 +648,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10336680" y="454680"/>
-          <a:ext cx="96840" cy="94320"/>
+          <a:ext cx="96120" cy="93600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -837,7 +843,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O103"/>
+  <dimension ref="A1:P103"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.33"/>
@@ -852,7 +858,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="23.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="29.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="29.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -900,6 +906,9 @@
       </c>
       <c r="O1" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -916,6 +925,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
@@ -926,16 +936,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5</v>
@@ -947,323 +957,426 @@
         <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O3" s="5" t="n">
         <v>45095</v>
       </c>
+      <c r="P3" s="1" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O22" s="5"/>
+      <c r="P22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O23" s="5"/>
+      <c r="P23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O26" s="5"/>
+      <c r="P26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O27" s="5"/>
+      <c r="P27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O28" s="5"/>
+      <c r="P28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O30" s="5"/>
+      <c r="P30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O31" s="5"/>
+      <c r="P31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O32" s="5"/>
+      <c r="P32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O34" s="5"/>
+      <c r="P34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O35" s="5"/>
+      <c r="P35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O36" s="5"/>
+      <c r="P36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O37" s="5"/>
+      <c r="P37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O38" s="5"/>
+      <c r="P38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O39" s="5"/>
+      <c r="P39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O40" s="5"/>
+      <c r="P40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O41" s="5"/>
+      <c r="P41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O42" s="5"/>
+      <c r="P42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O43" s="5"/>
+      <c r="P43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O44" s="5"/>
+      <c r="P44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O45" s="5"/>
+      <c r="P45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O46" s="5"/>
+      <c r="P46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O47" s="5"/>
+      <c r="P47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O48" s="5"/>
+      <c r="P48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O49" s="5"/>
+      <c r="P49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O50" s="5"/>
+      <c r="P50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O51" s="5"/>
+      <c r="P51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O52" s="5"/>
+      <c r="P52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O53" s="5"/>
+      <c r="P53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O54" s="5"/>
+      <c r="P54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O55" s="5"/>
+      <c r="P55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O56" s="5"/>
+      <c r="P56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O57" s="5"/>
+      <c r="P57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O58" s="5"/>
+      <c r="P58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O59" s="5"/>
+      <c r="P59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O60" s="5"/>
+      <c r="P60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O61" s="5"/>
+      <c r="P61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O62" s="5"/>
+      <c r="P62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O63" s="5"/>
+      <c r="P63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O64" s="5"/>
+      <c r="P64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O65" s="5"/>
+      <c r="P65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O66" s="5"/>
+      <c r="P66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O67" s="5"/>
+      <c r="P67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O68" s="5"/>
+      <c r="P68" s="5"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O69" s="5"/>
+      <c r="P69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O70" s="5"/>
+      <c r="P70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O71" s="5"/>
+      <c r="P71" s="5"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O72" s="5"/>
+      <c r="P72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O73" s="5"/>
+      <c r="P73" s="5"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O74" s="5"/>
+      <c r="P74" s="5"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O75" s="5"/>
+      <c r="P75" s="5"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O76" s="5"/>
+      <c r="P76" s="5"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O77" s="5"/>
+      <c r="P77" s="5"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O78" s="5"/>
+      <c r="P78" s="5"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O79" s="5"/>
+      <c r="P79" s="5"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O80" s="5"/>
+      <c r="P80" s="5"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O81" s="5"/>
+      <c r="P81" s="5"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O82" s="5"/>
+      <c r="P82" s="5"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O83" s="5"/>
+      <c r="P83" s="5"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O84" s="5"/>
+      <c r="P84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O85" s="5"/>
+      <c r="P85" s="5"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O86" s="5"/>
+      <c r="P86" s="5"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O87" s="5"/>
+      <c r="P87" s="5"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O88" s="5"/>
+      <c r="P88" s="5"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O89" s="5"/>
+      <c r="P89" s="5"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O90" s="5"/>
+      <c r="P90" s="5"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O91" s="5"/>
+      <c r="P91" s="5"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O92" s="5"/>
+      <c r="P92" s="5"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O93" s="5"/>
+      <c r="P93" s="5"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O94" s="5"/>
+      <c r="P94" s="5"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O95" s="5"/>
+      <c r="P95" s="5"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O96" s="5"/>
+      <c r="P96" s="5"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O97" s="5"/>
+      <c r="P97" s="5"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O98" s="5"/>
+      <c r="P98" s="5"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O99" s="5"/>
+      <c r="P99" s="5"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O100" s="5"/>
+      <c r="P100" s="5"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O101" s="5"/>
+      <c r="P101" s="5"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O102" s="5"/>
+      <c r="P102" s="5"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O103" s="5"/>
+      <c r="P103" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1281,86 +1394,89 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R371"/>
+  <dimension ref="A1:S1048576"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="19.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="19.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="11.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="35.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="13.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="17.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="21.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="19.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="18.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="19.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="11.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="C1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -1378,1672 +1494,1643 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>39</v>
+      <c r="B3" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="G3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="5" t="n">
         <v>28558</v>
       </c>
-      <c r="J3" s="4" t="b">
+      <c r="K3" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>15</v>
+      <c r="L3" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="O3" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="P3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q3" s="5" t="n">
+      <c r="R3" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R3" s="6" t="s">
-        <v>47</v>
+      <c r="S3" s="6" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I4" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J4" s="5" t="n">
         <v>24971</v>
       </c>
-      <c r="J4" s="4" t="b">
+      <c r="K4" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="Q4" s="5" t="n">
+      <c r="R4" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R4" s="6" t="s">
-        <v>52</v>
+      <c r="S4" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I5" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J5" s="5" t="n">
         <v>24092</v>
       </c>
-      <c r="J5" s="4" t="b">
+      <c r="K5" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K5" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="P5" s="1" t="n">
+      <c r="L5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q5" s="5" t="n">
+      <c r="R5" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R5" s="6" t="s">
-        <v>52</v>
+      <c r="S5" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="C6" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I6" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="5" t="n">
         <v>43298</v>
       </c>
-      <c r="J6" s="4" t="b">
+      <c r="K6" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q6" s="5" t="n">
+      <c r="L6" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="R6" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R6" s="6" t="s">
-        <v>52</v>
+      <c r="S6" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I7" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J7" s="5" t="n">
         <v>34615</v>
       </c>
-      <c r="J7" s="4" t="b">
+      <c r="K7" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="Q7" s="5" t="n">
+      <c r="R7" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R7" s="6" t="s">
-        <v>52</v>
+      <c r="S7" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I8" s="5"/>
-      <c r="Q8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="R8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I9" s="5"/>
-      <c r="Q9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="R9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I10" s="5"/>
-      <c r="Q10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="R10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I11" s="5"/>
-      <c r="Q11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="R11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I12" s="5"/>
-      <c r="Q12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="R12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I13" s="5"/>
-      <c r="Q13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="R13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I14" s="5"/>
-      <c r="Q14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="R14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I15" s="5"/>
-      <c r="Q15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="R15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I16" s="5"/>
-      <c r="Q16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="R16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I17" s="5"/>
-      <c r="Q17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="R17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I18" s="5"/>
-      <c r="Q18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="R18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I19" s="5"/>
-      <c r="Q19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="R19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I20" s="5"/>
-      <c r="Q20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="R20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I21" s="5"/>
-      <c r="Q21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="R21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I22" s="5"/>
-      <c r="Q22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="R22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I23" s="5"/>
-      <c r="Q23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="R23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I24" s="5"/>
-      <c r="Q24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="R24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I25" s="5"/>
-      <c r="Q25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="R25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I26" s="5"/>
-      <c r="Q26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="R26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I27" s="5"/>
-      <c r="Q27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="R27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I28" s="5"/>
-      <c r="Q28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="R28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I29" s="5"/>
-      <c r="Q29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="R29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I30" s="5"/>
-      <c r="Q30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="R30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I31" s="5"/>
-      <c r="Q31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="R31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I32" s="5"/>
-      <c r="Q32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="R32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I33" s="5"/>
-      <c r="Q33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="R33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I34" s="5"/>
-      <c r="Q34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="R34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I35" s="5"/>
-      <c r="Q35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="R35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I36" s="5"/>
-      <c r="Q36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="R36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I37" s="5"/>
-      <c r="Q37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="R37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I38" s="5"/>
-      <c r="Q38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="R38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I39" s="5"/>
-      <c r="Q39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="R39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I40" s="5"/>
-      <c r="Q40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="R40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I41" s="5"/>
-      <c r="Q41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="R41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I42" s="5"/>
-      <c r="Q42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="R42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I43" s="5"/>
-      <c r="Q43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="R43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I44" s="5"/>
-      <c r="Q44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="R44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I45" s="5"/>
-      <c r="Q45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="R45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I46" s="5"/>
-      <c r="Q46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="R46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I47" s="5"/>
-      <c r="Q47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="R47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I48" s="5"/>
-      <c r="Q48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="R48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I49" s="5"/>
-      <c r="Q49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="R49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I50" s="5"/>
-      <c r="Q50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="R50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I51" s="5"/>
-      <c r="Q51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="R51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I52" s="5"/>
-      <c r="Q52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="R52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I53" s="5"/>
-      <c r="Q53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="R53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I54" s="5"/>
-      <c r="Q54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="R54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I55" s="5"/>
-      <c r="Q55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="R55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I56" s="5"/>
-      <c r="Q56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="R56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I57" s="5"/>
-      <c r="Q57" s="5"/>
+      <c r="J57" s="5"/>
+      <c r="R57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I58" s="5"/>
-      <c r="Q58" s="5"/>
+      <c r="J58" s="5"/>
+      <c r="R58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I59" s="5"/>
-      <c r="Q59" s="5"/>
+      <c r="J59" s="5"/>
+      <c r="R59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I60" s="5"/>
-      <c r="Q60" s="5"/>
+      <c r="J60" s="5"/>
+      <c r="R60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I61" s="5"/>
-      <c r="Q61" s="5"/>
+      <c r="J61" s="5"/>
+      <c r="R61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I62" s="5"/>
-      <c r="Q62" s="5"/>
+      <c r="J62" s="5"/>
+      <c r="R62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I63" s="5"/>
-      <c r="Q63" s="5"/>
+      <c r="J63" s="5"/>
+      <c r="R63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I64" s="5"/>
-      <c r="Q64" s="5"/>
+      <c r="J64" s="5"/>
+      <c r="R64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I65" s="5"/>
-      <c r="Q65" s="5"/>
+      <c r="J65" s="5"/>
+      <c r="R65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I66" s="5"/>
-      <c r="Q66" s="5"/>
+      <c r="J66" s="5"/>
+      <c r="R66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I67" s="5"/>
-      <c r="Q67" s="5"/>
+      <c r="J67" s="5"/>
+      <c r="R67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I68" s="5"/>
-      <c r="Q68" s="5"/>
+      <c r="J68" s="5"/>
+      <c r="R68" s="5"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I69" s="5"/>
-      <c r="Q69" s="5"/>
+      <c r="J69" s="5"/>
+      <c r="R69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I70" s="5"/>
-      <c r="Q70" s="5"/>
+      <c r="J70" s="5"/>
+      <c r="R70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I71" s="5"/>
-      <c r="Q71" s="5"/>
+      <c r="J71" s="5"/>
+      <c r="R71" s="5"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I72" s="5"/>
-      <c r="Q72" s="5"/>
+      <c r="J72" s="5"/>
+      <c r="R72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I73" s="5"/>
-      <c r="Q73" s="5"/>
+      <c r="J73" s="5"/>
+      <c r="R73" s="5"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I74" s="5"/>
-      <c r="Q74" s="5"/>
+      <c r="J74" s="5"/>
+      <c r="R74" s="5"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I75" s="5"/>
-      <c r="Q75" s="5"/>
+      <c r="J75" s="5"/>
+      <c r="R75" s="5"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I76" s="5"/>
-      <c r="Q76" s="5"/>
+      <c r="J76" s="5"/>
+      <c r="R76" s="5"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I77" s="5"/>
-      <c r="Q77" s="5"/>
+      <c r="J77" s="5"/>
+      <c r="R77" s="5"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I78" s="5"/>
-      <c r="Q78" s="5"/>
+      <c r="J78" s="5"/>
+      <c r="R78" s="5"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I79" s="5"/>
-      <c r="Q79" s="5"/>
+      <c r="J79" s="5"/>
+      <c r="R79" s="5"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I80" s="5"/>
-      <c r="Q80" s="5"/>
+      <c r="J80" s="5"/>
+      <c r="R80" s="5"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I81" s="5"/>
-      <c r="Q81" s="5"/>
+      <c r="J81" s="5"/>
+      <c r="R81" s="5"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I82" s="5"/>
-      <c r="Q82" s="5"/>
+      <c r="J82" s="5"/>
+      <c r="R82" s="5"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I83" s="5"/>
-      <c r="Q83" s="5"/>
+      <c r="J83" s="5"/>
+      <c r="R83" s="5"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I84" s="5"/>
-      <c r="Q84" s="5"/>
+      <c r="J84" s="5"/>
+      <c r="R84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I85" s="5"/>
-      <c r="Q85" s="5"/>
+      <c r="J85" s="5"/>
+      <c r="R85" s="5"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I86" s="5"/>
-      <c r="Q86" s="5"/>
+      <c r="J86" s="5"/>
+      <c r="R86" s="5"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I87" s="5"/>
-      <c r="Q87" s="5"/>
+      <c r="J87" s="5"/>
+      <c r="R87" s="5"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I88" s="5"/>
-      <c r="Q88" s="5"/>
+      <c r="J88" s="5"/>
+      <c r="R88" s="5"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I89" s="5"/>
-      <c r="Q89" s="5"/>
+      <c r="J89" s="5"/>
+      <c r="R89" s="5"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I90" s="5"/>
-      <c r="Q90" s="5"/>
+      <c r="J90" s="5"/>
+      <c r="R90" s="5"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I91" s="5"/>
-      <c r="Q91" s="5"/>
+      <c r="J91" s="5"/>
+      <c r="R91" s="5"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I92" s="5"/>
-      <c r="Q92" s="5"/>
+      <c r="J92" s="5"/>
+      <c r="R92" s="5"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I93" s="5"/>
-      <c r="Q93" s="5"/>
+      <c r="J93" s="5"/>
+      <c r="R93" s="5"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I94" s="5"/>
-      <c r="Q94" s="5"/>
+      <c r="J94" s="5"/>
+      <c r="R94" s="5"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I95" s="5"/>
-      <c r="Q95" s="5"/>
+      <c r="J95" s="5"/>
+      <c r="R95" s="5"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I96" s="5"/>
-      <c r="Q96" s="5"/>
+      <c r="J96" s="5"/>
+      <c r="R96" s="5"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I97" s="5"/>
-      <c r="Q97" s="5"/>
+      <c r="J97" s="5"/>
+      <c r="R97" s="5"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I98" s="5"/>
-      <c r="Q98" s="5"/>
+      <c r="J98" s="5"/>
+      <c r="R98" s="5"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I99" s="5"/>
-      <c r="Q99" s="5"/>
+      <c r="J99" s="5"/>
+      <c r="R99" s="5"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I100" s="5"/>
-      <c r="Q100" s="5"/>
+      <c r="J100" s="5"/>
+      <c r="R100" s="5"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I101" s="5"/>
-      <c r="Q101" s="5"/>
+      <c r="J101" s="5"/>
+      <c r="R101" s="5"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I102" s="5"/>
-      <c r="Q102" s="5"/>
+      <c r="J102" s="5"/>
+      <c r="R102" s="5"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I103" s="5"/>
-      <c r="Q103" s="5"/>
+      <c r="J103" s="5"/>
+      <c r="R103" s="5"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I104" s="5"/>
-      <c r="Q104" s="5"/>
+      <c r="J104" s="5"/>
+      <c r="R104" s="5"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I105" s="5"/>
-      <c r="Q105" s="5"/>
+      <c r="J105" s="5"/>
+      <c r="R105" s="5"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I106" s="5"/>
-      <c r="Q106" s="5"/>
+      <c r="J106" s="5"/>
+      <c r="R106" s="5"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I107" s="5"/>
-      <c r="Q107" s="5"/>
+      <c r="J107" s="5"/>
+      <c r="R107" s="5"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I108" s="5"/>
-      <c r="Q108" s="5"/>
+      <c r="J108" s="5"/>
+      <c r="R108" s="5"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I109" s="5"/>
-      <c r="Q109" s="5"/>
+      <c r="J109" s="5"/>
+      <c r="R109" s="5"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I110" s="5"/>
-      <c r="Q110" s="5"/>
+      <c r="J110" s="5"/>
+      <c r="R110" s="5"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I111" s="5"/>
-      <c r="Q111" s="5"/>
+      <c r="J111" s="5"/>
+      <c r="R111" s="5"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I112" s="5"/>
-      <c r="Q112" s="5"/>
+      <c r="J112" s="5"/>
+      <c r="R112" s="5"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I113" s="5"/>
-      <c r="Q113" s="5"/>
+      <c r="J113" s="5"/>
+      <c r="R113" s="5"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I114" s="5"/>
-      <c r="Q114" s="5"/>
+      <c r="J114" s="5"/>
+      <c r="R114" s="5"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I115" s="5"/>
-      <c r="Q115" s="5"/>
+      <c r="J115" s="5"/>
+      <c r="R115" s="5"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I116" s="5"/>
-      <c r="Q116" s="5"/>
+      <c r="J116" s="5"/>
+      <c r="R116" s="5"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I117" s="5"/>
-      <c r="Q117" s="5"/>
+      <c r="J117" s="5"/>
+      <c r="R117" s="5"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I118" s="5"/>
-      <c r="Q118" s="5"/>
+      <c r="J118" s="5"/>
+      <c r="R118" s="5"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I119" s="5"/>
-      <c r="Q119" s="5"/>
+      <c r="J119" s="5"/>
+      <c r="R119" s="5"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I120" s="5"/>
-      <c r="Q120" s="5"/>
+      <c r="J120" s="5"/>
+      <c r="R120" s="5"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I121" s="5"/>
-      <c r="Q121" s="5"/>
+      <c r="J121" s="5"/>
+      <c r="R121" s="5"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I122" s="5"/>
-      <c r="Q122" s="5"/>
+      <c r="J122" s="5"/>
+      <c r="R122" s="5"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I123" s="5"/>
-      <c r="Q123" s="5"/>
+      <c r="J123" s="5"/>
+      <c r="R123" s="5"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I124" s="5"/>
-      <c r="Q124" s="5"/>
+      <c r="J124" s="5"/>
+      <c r="R124" s="5"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I125" s="5"/>
-      <c r="Q125" s="5"/>
+      <c r="J125" s="5"/>
+      <c r="R125" s="5"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I126" s="5"/>
-      <c r="Q126" s="5"/>
+      <c r="J126" s="5"/>
+      <c r="R126" s="5"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I127" s="5"/>
-      <c r="Q127" s="5"/>
+      <c r="J127" s="5"/>
+      <c r="R127" s="5"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I128" s="5"/>
-      <c r="Q128" s="5"/>
+      <c r="J128" s="5"/>
+      <c r="R128" s="5"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I129" s="5"/>
-      <c r="Q129" s="5"/>
+      <c r="J129" s="5"/>
+      <c r="R129" s="5"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I130" s="5"/>
-      <c r="Q130" s="5"/>
+      <c r="J130" s="5"/>
+      <c r="R130" s="5"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I131" s="5"/>
-      <c r="Q131" s="5"/>
+      <c r="J131" s="5"/>
+      <c r="R131" s="5"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I132" s="5"/>
-      <c r="Q132" s="5"/>
+      <c r="J132" s="5"/>
+      <c r="R132" s="5"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I133" s="5"/>
-      <c r="Q133" s="5"/>
+      <c r="J133" s="5"/>
+      <c r="R133" s="5"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I134" s="5"/>
-      <c r="Q134" s="5"/>
+      <c r="J134" s="5"/>
+      <c r="R134" s="5"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I135" s="5"/>
-      <c r="Q135" s="5"/>
+      <c r="J135" s="5"/>
+      <c r="R135" s="5"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I136" s="5"/>
-      <c r="Q136" s="5"/>
+      <c r="J136" s="5"/>
+      <c r="R136" s="5"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I137" s="5"/>
-      <c r="Q137" s="5"/>
+      <c r="J137" s="5"/>
+      <c r="R137" s="5"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I138" s="5"/>
-      <c r="Q138" s="5"/>
+      <c r="J138" s="5"/>
+      <c r="R138" s="5"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I139" s="5"/>
-      <c r="Q139" s="5"/>
+      <c r="J139" s="5"/>
+      <c r="R139" s="5"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I140" s="5"/>
-      <c r="Q140" s="5"/>
+      <c r="J140" s="5"/>
+      <c r="R140" s="5"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I141" s="5"/>
-      <c r="Q141" s="5"/>
+      <c r="J141" s="5"/>
+      <c r="R141" s="5"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I142" s="5"/>
-      <c r="Q142" s="5"/>
+      <c r="J142" s="5"/>
+      <c r="R142" s="5"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I143" s="5"/>
-      <c r="Q143" s="5"/>
+      <c r="J143" s="5"/>
+      <c r="R143" s="5"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I144" s="5"/>
-      <c r="Q144" s="5"/>
+      <c r="J144" s="5"/>
+      <c r="R144" s="5"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I145" s="5"/>
-      <c r="Q145" s="5"/>
+      <c r="J145" s="5"/>
+      <c r="R145" s="5"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I146" s="5"/>
-      <c r="Q146" s="5"/>
+      <c r="J146" s="5"/>
+      <c r="R146" s="5"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I147" s="5"/>
-      <c r="Q147" s="5"/>
+      <c r="J147" s="5"/>
+      <c r="R147" s="5"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I148" s="5"/>
-      <c r="Q148" s="5"/>
+      <c r="J148" s="5"/>
+      <c r="R148" s="5"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I149" s="5"/>
-      <c r="Q149" s="5"/>
+      <c r="J149" s="5"/>
+      <c r="R149" s="5"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I150" s="5"/>
-      <c r="Q150" s="5"/>
+      <c r="J150" s="5"/>
+      <c r="R150" s="5"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I151" s="5"/>
-      <c r="Q151" s="5"/>
+      <c r="J151" s="5"/>
+      <c r="R151" s="5"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I152" s="5"/>
-      <c r="Q152" s="5"/>
+      <c r="J152" s="5"/>
+      <c r="R152" s="5"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I153" s="5"/>
-      <c r="Q153" s="5"/>
+      <c r="J153" s="5"/>
+      <c r="R153" s="5"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I154" s="5"/>
-      <c r="Q154" s="5"/>
+      <c r="J154" s="5"/>
+      <c r="R154" s="5"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I155" s="5"/>
-      <c r="Q155" s="5"/>
+      <c r="J155" s="5"/>
+      <c r="R155" s="5"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I156" s="5"/>
-      <c r="Q156" s="5"/>
+      <c r="J156" s="5"/>
+      <c r="R156" s="5"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I157" s="5"/>
-      <c r="Q157" s="5"/>
+      <c r="J157" s="5"/>
+      <c r="R157" s="5"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I158" s="5"/>
-      <c r="Q158" s="5"/>
+      <c r="J158" s="5"/>
+      <c r="R158" s="5"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I159" s="5"/>
-      <c r="Q159" s="5"/>
+      <c r="J159" s="5"/>
+      <c r="R159" s="5"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I160" s="5"/>
-      <c r="Q160" s="5"/>
+      <c r="J160" s="5"/>
+      <c r="R160" s="5"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I161" s="5"/>
-      <c r="Q161" s="5"/>
+      <c r="J161" s="5"/>
+      <c r="R161" s="5"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I162" s="5"/>
-      <c r="Q162" s="5"/>
+      <c r="J162" s="5"/>
+      <c r="R162" s="5"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I163" s="5"/>
-      <c r="Q163" s="5"/>
+      <c r="J163" s="5"/>
+      <c r="R163" s="5"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I164" s="5"/>
-      <c r="Q164" s="5"/>
+      <c r="J164" s="5"/>
+      <c r="R164" s="5"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I165" s="5"/>
-      <c r="Q165" s="5"/>
+      <c r="J165" s="5"/>
+      <c r="R165" s="5"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I166" s="5"/>
-      <c r="Q166" s="5"/>
+      <c r="J166" s="5"/>
+      <c r="R166" s="5"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I167" s="5"/>
-      <c r="Q167" s="5"/>
+      <c r="J167" s="5"/>
+      <c r="R167" s="5"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I168" s="5"/>
-      <c r="Q168" s="5"/>
+      <c r="J168" s="5"/>
+      <c r="R168" s="5"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I169" s="5"/>
-      <c r="Q169" s="5"/>
+      <c r="J169" s="5"/>
+      <c r="R169" s="5"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I170" s="5"/>
-      <c r="Q170" s="5"/>
+      <c r="J170" s="5"/>
+      <c r="R170" s="5"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I171" s="5"/>
-      <c r="Q171" s="5"/>
+      <c r="J171" s="5"/>
+      <c r="R171" s="5"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I172" s="5"/>
-      <c r="Q172" s="5"/>
+      <c r="J172" s="5"/>
+      <c r="R172" s="5"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I173" s="5"/>
-      <c r="Q173" s="5"/>
+      <c r="J173" s="5"/>
+      <c r="R173" s="5"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I174" s="5"/>
-      <c r="Q174" s="5"/>
+      <c r="J174" s="5"/>
+      <c r="R174" s="5"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I175" s="5"/>
-      <c r="Q175" s="5"/>
+      <c r="J175" s="5"/>
+      <c r="R175" s="5"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I176" s="5"/>
-      <c r="Q176" s="5"/>
+      <c r="J176" s="5"/>
+      <c r="R176" s="5"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I177" s="5"/>
-      <c r="Q177" s="5"/>
+      <c r="J177" s="5"/>
+      <c r="R177" s="5"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I178" s="5"/>
-      <c r="Q178" s="5"/>
+      <c r="J178" s="5"/>
+      <c r="R178" s="5"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I179" s="5"/>
-      <c r="Q179" s="5"/>
+      <c r="J179" s="5"/>
+      <c r="R179" s="5"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I180" s="5"/>
-      <c r="Q180" s="5"/>
+      <c r="J180" s="5"/>
+      <c r="R180" s="5"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I181" s="5"/>
-      <c r="Q181" s="5"/>
+      <c r="J181" s="5"/>
+      <c r="R181" s="5"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I182" s="5"/>
-      <c r="Q182" s="5"/>
+      <c r="J182" s="5"/>
+      <c r="R182" s="5"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I183" s="5"/>
-      <c r="Q183" s="5"/>
+      <c r="J183" s="5"/>
+      <c r="R183" s="5"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I184" s="5"/>
-      <c r="Q184" s="5"/>
+      <c r="J184" s="5"/>
+      <c r="R184" s="5"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I185" s="5"/>
-      <c r="Q185" s="5"/>
+      <c r="J185" s="5"/>
+      <c r="R185" s="5"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I186" s="5"/>
-      <c r="Q186" s="5"/>
+      <c r="J186" s="5"/>
+      <c r="R186" s="5"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I187" s="5"/>
-      <c r="Q187" s="5"/>
+      <c r="J187" s="5"/>
+      <c r="R187" s="5"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I188" s="5"/>
-      <c r="Q188" s="5"/>
+      <c r="J188" s="5"/>
+      <c r="R188" s="5"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I189" s="5"/>
-      <c r="Q189" s="5"/>
+      <c r="J189" s="5"/>
+      <c r="R189" s="5"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I190" s="5"/>
-      <c r="Q190" s="5"/>
+      <c r="J190" s="5"/>
+      <c r="R190" s="5"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I191" s="5"/>
-      <c r="Q191" s="5"/>
+      <c r="J191" s="5"/>
+      <c r="R191" s="5"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I192" s="5"/>
-      <c r="Q192" s="5"/>
+      <c r="J192" s="5"/>
+      <c r="R192" s="5"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I193" s="5"/>
-      <c r="Q193" s="5"/>
+      <c r="J193" s="5"/>
+      <c r="R193" s="5"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I194" s="5"/>
-      <c r="Q194" s="5"/>
+      <c r="J194" s="5"/>
+      <c r="R194" s="5"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I195" s="5"/>
-      <c r="Q195" s="5"/>
+      <c r="J195" s="5"/>
+      <c r="R195" s="5"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I196" s="5"/>
-      <c r="Q196" s="5"/>
+      <c r="J196" s="5"/>
+      <c r="R196" s="5"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I197" s="5"/>
-      <c r="Q197" s="5"/>
+      <c r="J197" s="5"/>
+      <c r="R197" s="5"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I198" s="5"/>
-      <c r="Q198" s="5"/>
+      <c r="J198" s="5"/>
+      <c r="R198" s="5"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I199" s="5"/>
-      <c r="Q199" s="5"/>
+      <c r="J199" s="5"/>
+      <c r="R199" s="5"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I200" s="5"/>
-      <c r="Q200" s="5"/>
+      <c r="J200" s="5"/>
+      <c r="R200" s="5"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I201" s="5"/>
-      <c r="Q201" s="5"/>
+      <c r="J201" s="5"/>
+      <c r="R201" s="5"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I202" s="5"/>
-      <c r="Q202" s="5"/>
+      <c r="J202" s="5"/>
+      <c r="R202" s="5"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I203" s="5"/>
-      <c r="Q203" s="5"/>
+      <c r="J203" s="5"/>
+      <c r="R203" s="5"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I204" s="5"/>
-      <c r="Q204" s="5"/>
+      <c r="J204" s="5"/>
+      <c r="R204" s="5"/>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I205" s="5"/>
-      <c r="Q205" s="5"/>
+      <c r="J205" s="5"/>
+      <c r="R205" s="5"/>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I206" s="5"/>
-      <c r="Q206" s="5"/>
+      <c r="J206" s="5"/>
+      <c r="R206" s="5"/>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I207" s="5"/>
-      <c r="Q207" s="5"/>
+      <c r="J207" s="5"/>
+      <c r="R207" s="5"/>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I208" s="5"/>
-      <c r="Q208" s="5"/>
+      <c r="J208" s="5"/>
+      <c r="R208" s="5"/>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I209" s="5"/>
-      <c r="Q209" s="5"/>
+      <c r="J209" s="5"/>
+      <c r="R209" s="5"/>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I210" s="5"/>
-      <c r="Q210" s="5"/>
+      <c r="J210" s="5"/>
+      <c r="R210" s="5"/>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I211" s="5"/>
-      <c r="Q211" s="5"/>
+      <c r="J211" s="5"/>
+      <c r="R211" s="5"/>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I212" s="5"/>
-      <c r="Q212" s="5"/>
+      <c r="J212" s="5"/>
+      <c r="R212" s="5"/>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I213" s="5"/>
-      <c r="Q213" s="5"/>
+      <c r="J213" s="5"/>
+      <c r="R213" s="5"/>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I214" s="5"/>
-      <c r="Q214" s="5"/>
+      <c r="J214" s="5"/>
+      <c r="R214" s="5"/>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I215" s="5"/>
-      <c r="Q215" s="5"/>
+      <c r="J215" s="5"/>
+      <c r="R215" s="5"/>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I216" s="5"/>
-      <c r="Q216" s="5"/>
+      <c r="J216" s="5"/>
+      <c r="R216" s="5"/>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I217" s="5"/>
-      <c r="Q217" s="5"/>
+      <c r="J217" s="5"/>
+      <c r="R217" s="5"/>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I218" s="5"/>
-      <c r="Q218" s="5"/>
+      <c r="J218" s="5"/>
+      <c r="R218" s="5"/>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I219" s="5"/>
-      <c r="Q219" s="5"/>
+      <c r="J219" s="5"/>
+      <c r="R219" s="5"/>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I220" s="5"/>
-      <c r="Q220" s="5"/>
+      <c r="J220" s="5"/>
+      <c r="R220" s="5"/>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I221" s="5"/>
-      <c r="Q221" s="5"/>
+      <c r="J221" s="5"/>
+      <c r="R221" s="5"/>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I222" s="5"/>
-      <c r="Q222" s="5"/>
+      <c r="J222" s="5"/>
+      <c r="R222" s="5"/>
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I223" s="5"/>
-      <c r="Q223" s="5"/>
+      <c r="J223" s="5"/>
+      <c r="R223" s="5"/>
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I224" s="5"/>
-      <c r="Q224" s="5"/>
+      <c r="J224" s="5"/>
+      <c r="R224" s="5"/>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I225" s="5"/>
-      <c r="Q225" s="5"/>
+      <c r="J225" s="5"/>
+      <c r="R225" s="5"/>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I226" s="5"/>
-      <c r="Q226" s="5"/>
+      <c r="J226" s="5"/>
+      <c r="R226" s="5"/>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I227" s="5"/>
-      <c r="Q227" s="5"/>
+      <c r="J227" s="5"/>
+      <c r="R227" s="5"/>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I228" s="5"/>
-      <c r="Q228" s="5"/>
+      <c r="J228" s="5"/>
+      <c r="R228" s="5"/>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I229" s="5"/>
-      <c r="Q229" s="5"/>
+      <c r="J229" s="5"/>
+      <c r="R229" s="5"/>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I230" s="5"/>
-      <c r="Q230" s="5"/>
+      <c r="J230" s="5"/>
+      <c r="R230" s="5"/>
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I231" s="5"/>
-      <c r="Q231" s="5"/>
+      <c r="J231" s="5"/>
+      <c r="R231" s="5"/>
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I232" s="5"/>
-      <c r="Q232" s="5"/>
+      <c r="J232" s="5"/>
+      <c r="R232" s="5"/>
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I233" s="5"/>
-      <c r="Q233" s="5"/>
+      <c r="J233" s="5"/>
+      <c r="R233" s="5"/>
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I234" s="5"/>
-      <c r="Q234" s="5"/>
+      <c r="J234" s="5"/>
+      <c r="R234" s="5"/>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I235" s="5"/>
-      <c r="Q235" s="5"/>
+      <c r="J235" s="5"/>
+      <c r="R235" s="5"/>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I236" s="5"/>
-      <c r="Q236" s="5"/>
+      <c r="J236" s="5"/>
+      <c r="R236" s="5"/>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I237" s="5"/>
-      <c r="Q237" s="5"/>
+      <c r="J237" s="5"/>
+      <c r="R237" s="5"/>
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I238" s="5"/>
-      <c r="Q238" s="5"/>
+      <c r="J238" s="5"/>
+      <c r="R238" s="5"/>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I239" s="5"/>
-      <c r="Q239" s="5"/>
+      <c r="J239" s="5"/>
+      <c r="R239" s="5"/>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I240" s="5"/>
-      <c r="Q240" s="5"/>
+      <c r="J240" s="5"/>
+      <c r="R240" s="5"/>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I241" s="5"/>
-      <c r="Q241" s="5"/>
+      <c r="J241" s="5"/>
+      <c r="R241" s="5"/>
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I242" s="5"/>
-      <c r="Q242" s="5"/>
+      <c r="J242" s="5"/>
+      <c r="R242" s="5"/>
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I243" s="5"/>
-      <c r="Q243" s="5"/>
+      <c r="J243" s="5"/>
+      <c r="R243" s="5"/>
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I244" s="5"/>
-      <c r="Q244" s="5"/>
+      <c r="J244" s="5"/>
+      <c r="R244" s="5"/>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I245" s="5"/>
-      <c r="Q245" s="5"/>
+      <c r="J245" s="5"/>
+      <c r="R245" s="5"/>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I246" s="5"/>
-      <c r="Q246" s="5"/>
+      <c r="J246" s="5"/>
+      <c r="R246" s="5"/>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I247" s="5"/>
-      <c r="Q247" s="5"/>
+      <c r="J247" s="5"/>
+      <c r="R247" s="5"/>
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I248" s="5"/>
-      <c r="Q248" s="5"/>
+      <c r="J248" s="5"/>
+      <c r="R248" s="5"/>
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I249" s="5"/>
-      <c r="Q249" s="5"/>
+      <c r="J249" s="5"/>
+      <c r="R249" s="5"/>
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I250" s="5"/>
-      <c r="Q250" s="5"/>
+      <c r="J250" s="5"/>
+      <c r="R250" s="5"/>
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I251" s="5"/>
-      <c r="Q251" s="5"/>
+      <c r="J251" s="5"/>
+      <c r="R251" s="5"/>
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I252" s="5"/>
-      <c r="Q252" s="5"/>
+      <c r="J252" s="5"/>
+      <c r="R252" s="5"/>
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I253" s="5"/>
-      <c r="Q253" s="5"/>
+      <c r="J253" s="5"/>
+      <c r="R253" s="5"/>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I254" s="5"/>
-      <c r="Q254" s="5"/>
+      <c r="J254" s="5"/>
+      <c r="R254" s="5"/>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I255" s="5"/>
-      <c r="Q255" s="5"/>
+      <c r="J255" s="5"/>
+      <c r="R255" s="5"/>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I256" s="5"/>
-      <c r="Q256" s="5"/>
+      <c r="J256" s="5"/>
+      <c r="R256" s="5"/>
     </row>
     <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I257" s="5"/>
-      <c r="Q257" s="5"/>
+      <c r="J257" s="5"/>
+      <c r="R257" s="5"/>
     </row>
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I258" s="5"/>
-      <c r="Q258" s="5"/>
+      <c r="J258" s="5"/>
+      <c r="R258" s="5"/>
     </row>
     <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I259" s="5"/>
-      <c r="Q259" s="5"/>
+      <c r="J259" s="5"/>
+      <c r="R259" s="5"/>
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I260" s="5"/>
-      <c r="Q260" s="5"/>
+      <c r="J260" s="5"/>
+      <c r="R260" s="5"/>
     </row>
     <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I261" s="5"/>
-      <c r="Q261" s="5"/>
+      <c r="J261" s="5"/>
+      <c r="R261" s="5"/>
     </row>
     <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I262" s="5"/>
-      <c r="Q262" s="5"/>
+      <c r="J262" s="5"/>
+      <c r="R262" s="5"/>
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I263" s="5"/>
-      <c r="Q263" s="5"/>
+      <c r="J263" s="5"/>
+      <c r="R263" s="5"/>
     </row>
     <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I264" s="5"/>
-      <c r="Q264" s="5"/>
+      <c r="J264" s="5"/>
+      <c r="R264" s="5"/>
     </row>
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I265" s="5"/>
-      <c r="Q265" s="5"/>
+      <c r="J265" s="5"/>
+      <c r="R265" s="5"/>
     </row>
     <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I266" s="5"/>
-      <c r="Q266" s="5"/>
+      <c r="J266" s="5"/>
+      <c r="R266" s="5"/>
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I267" s="5"/>
-      <c r="Q267" s="5"/>
+      <c r="J267" s="5"/>
+      <c r="R267" s="5"/>
     </row>
     <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I268" s="5"/>
-      <c r="Q268" s="5"/>
+      <c r="J268" s="5"/>
+      <c r="R268" s="5"/>
     </row>
     <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I269" s="5"/>
-      <c r="Q269" s="5"/>
+      <c r="J269" s="5"/>
+      <c r="R269" s="5"/>
     </row>
     <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I270" s="5"/>
-      <c r="Q270" s="5"/>
+      <c r="J270" s="5"/>
+      <c r="R270" s="5"/>
     </row>
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I271" s="5"/>
-      <c r="Q271" s="5"/>
+      <c r="J271" s="5"/>
+      <c r="R271" s="5"/>
     </row>
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I272" s="5"/>
-      <c r="Q272" s="5"/>
+      <c r="J272" s="5"/>
+      <c r="R272" s="5"/>
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I273" s="5"/>
-      <c r="Q273" s="5"/>
+      <c r="J273" s="5"/>
+      <c r="R273" s="5"/>
     </row>
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I274" s="5"/>
-      <c r="Q274" s="5"/>
+      <c r="J274" s="5"/>
+      <c r="R274" s="5"/>
     </row>
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I275" s="5"/>
-      <c r="Q275" s="5"/>
+      <c r="J275" s="5"/>
+      <c r="R275" s="5"/>
     </row>
     <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I276" s="5"/>
-      <c r="Q276" s="5"/>
+      <c r="J276" s="5"/>
+      <c r="R276" s="5"/>
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I277" s="5"/>
-      <c r="Q277" s="5"/>
+      <c r="J277" s="5"/>
+      <c r="R277" s="5"/>
     </row>
     <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I278" s="5"/>
-      <c r="Q278" s="5"/>
+      <c r="J278" s="5"/>
+      <c r="R278" s="5"/>
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I279" s="5"/>
-      <c r="Q279" s="5"/>
+      <c r="J279" s="5"/>
+      <c r="R279" s="5"/>
     </row>
     <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I280" s="5"/>
-      <c r="Q280" s="5"/>
+      <c r="J280" s="5"/>
+      <c r="R280" s="5"/>
     </row>
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I281" s="5"/>
-      <c r="Q281" s="5"/>
+      <c r="J281" s="5"/>
+      <c r="R281" s="5"/>
     </row>
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I282" s="5"/>
-      <c r="Q282" s="5"/>
+      <c r="J282" s="5"/>
+      <c r="R282" s="5"/>
     </row>
     <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I283" s="5"/>
-      <c r="Q283" s="5"/>
+      <c r="J283" s="5"/>
+      <c r="R283" s="5"/>
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I284" s="5"/>
-      <c r="Q284" s="5"/>
+      <c r="J284" s="5"/>
+      <c r="R284" s="5"/>
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I285" s="5"/>
-      <c r="Q285" s="5"/>
+      <c r="J285" s="5"/>
+      <c r="R285" s="5"/>
     </row>
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I286" s="5"/>
-      <c r="Q286" s="5"/>
+      <c r="J286" s="5"/>
+      <c r="R286" s="5"/>
     </row>
     <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I287" s="5"/>
-      <c r="Q287" s="5"/>
+      <c r="J287" s="5"/>
+      <c r="R287" s="5"/>
     </row>
     <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I288" s="5"/>
-      <c r="Q288" s="5"/>
+      <c r="J288" s="5"/>
+      <c r="R288" s="5"/>
     </row>
     <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I289" s="5"/>
-      <c r="Q289" s="5"/>
+      <c r="J289" s="5"/>
+      <c r="R289" s="5"/>
     </row>
     <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I290" s="5"/>
-      <c r="Q290" s="5"/>
+      <c r="J290" s="5"/>
+      <c r="R290" s="5"/>
     </row>
     <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I291" s="5"/>
-      <c r="Q291" s="5"/>
+      <c r="J291" s="5"/>
+      <c r="R291" s="5"/>
     </row>
     <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I292" s="5"/>
-      <c r="Q292" s="5"/>
+      <c r="J292" s="5"/>
+      <c r="R292" s="5"/>
     </row>
     <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I293" s="5"/>
-      <c r="Q293" s="5"/>
+      <c r="J293" s="5"/>
+      <c r="R293" s="5"/>
     </row>
     <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I294" s="5"/>
-      <c r="Q294" s="5"/>
+      <c r="J294" s="5"/>
+      <c r="R294" s="5"/>
     </row>
     <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I295" s="5"/>
-      <c r="Q295" s="5"/>
+      <c r="J295" s="5"/>
+      <c r="R295" s="5"/>
     </row>
     <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I296" s="5"/>
-      <c r="Q296" s="5"/>
+      <c r="J296" s="5"/>
+      <c r="R296" s="5"/>
     </row>
     <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I297" s="5"/>
-      <c r="Q297" s="5"/>
+      <c r="J297" s="5"/>
+      <c r="R297" s="5"/>
     </row>
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I298" s="5"/>
-      <c r="Q298" s="5"/>
+      <c r="J298" s="5"/>
+      <c r="R298" s="5"/>
     </row>
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I299" s="5"/>
-      <c r="Q299" s="5"/>
+      <c r="J299" s="5"/>
+      <c r="R299" s="5"/>
     </row>
     <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I300" s="5"/>
-      <c r="Q300" s="5"/>
+      <c r="J300" s="5"/>
+      <c r="R300" s="5"/>
     </row>
     <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I301" s="5"/>
-      <c r="Q301" s="5"/>
+      <c r="J301" s="5"/>
+      <c r="R301" s="5"/>
     </row>
     <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I302" s="5"/>
-      <c r="Q302" s="5"/>
+      <c r="J302" s="5"/>
+      <c r="R302" s="5"/>
     </row>
     <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I303" s="5"/>
-      <c r="Q303" s="5"/>
+      <c r="J303" s="5"/>
+      <c r="R303" s="5"/>
     </row>
     <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I304" s="5"/>
-      <c r="Q304" s="5"/>
+      <c r="J304" s="5"/>
+      <c r="R304" s="5"/>
     </row>
     <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I305" s="5"/>
-      <c r="Q305" s="5"/>
+      <c r="J305" s="5"/>
+      <c r="R305" s="5"/>
     </row>
     <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I306" s="5"/>
-      <c r="Q306" s="5"/>
+      <c r="J306" s="5"/>
+      <c r="R306" s="5"/>
     </row>
     <row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I307" s="5"/>
-      <c r="Q307" s="5"/>
+      <c r="J307" s="5"/>
+      <c r="R307" s="5"/>
     </row>
     <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I308" s="5"/>
-      <c r="Q308" s="5"/>
+      <c r="J308" s="5"/>
+      <c r="R308" s="5"/>
     </row>
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I309" s="5"/>
-      <c r="Q309" s="5"/>
+      <c r="J309" s="5"/>
+      <c r="R309" s="5"/>
     </row>
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I310" s="5"/>
-      <c r="Q310" s="5"/>
+      <c r="J310" s="5"/>
+      <c r="R310" s="5"/>
     </row>
     <row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I311" s="5"/>
-      <c r="Q311" s="5"/>
+      <c r="J311" s="5"/>
+      <c r="R311" s="5"/>
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I312" s="5"/>
-      <c r="Q312" s="5"/>
+      <c r="J312" s="5"/>
+      <c r="R312" s="5"/>
     </row>
     <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I313" s="5"/>
-      <c r="Q313" s="5"/>
+      <c r="J313" s="5"/>
+      <c r="R313" s="5"/>
     </row>
     <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I314" s="5"/>
-      <c r="Q314" s="5"/>
+      <c r="J314" s="5"/>
+      <c r="R314" s="5"/>
     </row>
     <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I315" s="5"/>
-      <c r="Q315" s="5"/>
+      <c r="J315" s="5"/>
+      <c r="R315" s="5"/>
     </row>
     <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I316" s="5"/>
-      <c r="Q316" s="5"/>
+      <c r="J316" s="5"/>
+      <c r="R316" s="5"/>
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I317" s="5"/>
-      <c r="Q317" s="5"/>
+      <c r="J317" s="5"/>
+      <c r="R317" s="5"/>
     </row>
     <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I318" s="5"/>
-      <c r="Q318" s="5"/>
+      <c r="J318" s="5"/>
+      <c r="R318" s="5"/>
     </row>
     <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I319" s="5"/>
-      <c r="Q319" s="5"/>
+      <c r="J319" s="5"/>
+      <c r="R319" s="5"/>
     </row>
     <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I320" s="5"/>
-      <c r="Q320" s="5"/>
+      <c r="J320" s="5"/>
+      <c r="R320" s="5"/>
     </row>
     <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I321" s="5"/>
-      <c r="Q321" s="5"/>
+      <c r="J321" s="5"/>
+      <c r="R321" s="5"/>
     </row>
     <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I322" s="5"/>
-      <c r="Q322" s="5"/>
+      <c r="J322" s="5"/>
+      <c r="R322" s="5"/>
     </row>
     <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I323" s="5"/>
-      <c r="Q323" s="5"/>
+      <c r="J323" s="5"/>
+      <c r="R323" s="5"/>
     </row>
     <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I324" s="5"/>
-      <c r="Q324" s="5"/>
+      <c r="J324" s="5"/>
+      <c r="R324" s="5"/>
     </row>
     <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I325" s="5"/>
-      <c r="Q325" s="5"/>
+      <c r="J325" s="5"/>
+      <c r="R325" s="5"/>
     </row>
     <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I326" s="5"/>
-      <c r="Q326" s="5"/>
+      <c r="J326" s="5"/>
+      <c r="R326" s="5"/>
     </row>
     <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I327" s="5"/>
-      <c r="Q327" s="5"/>
+      <c r="J327" s="5"/>
+      <c r="R327" s="5"/>
     </row>
     <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I328" s="5"/>
-      <c r="Q328" s="5"/>
+      <c r="J328" s="5"/>
+      <c r="R328" s="5"/>
     </row>
     <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I329" s="5"/>
-      <c r="Q329" s="5"/>
+      <c r="J329" s="5"/>
+      <c r="R329" s="5"/>
     </row>
     <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I330" s="5"/>
-      <c r="Q330" s="5"/>
+      <c r="J330" s="5"/>
+      <c r="R330" s="5"/>
     </row>
     <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I331" s="5"/>
-      <c r="Q331" s="5"/>
+      <c r="J331" s="5"/>
+      <c r="R331" s="5"/>
     </row>
     <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I332" s="5"/>
-      <c r="Q332" s="5"/>
+      <c r="J332" s="5"/>
+      <c r="R332" s="5"/>
     </row>
     <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I333" s="5"/>
-      <c r="Q333" s="5"/>
+      <c r="J333" s="5"/>
+      <c r="R333" s="5"/>
     </row>
     <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I334" s="5"/>
-      <c r="Q334" s="5"/>
+      <c r="J334" s="5"/>
+      <c r="R334" s="5"/>
     </row>
     <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I335" s="5"/>
-      <c r="Q335" s="5"/>
+      <c r="J335" s="5"/>
+      <c r="R335" s="5"/>
     </row>
     <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I336" s="5"/>
-      <c r="Q336" s="5"/>
+      <c r="J336" s="5"/>
+      <c r="R336" s="5"/>
     </row>
     <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I337" s="5"/>
-      <c r="Q337" s="5"/>
+      <c r="J337" s="5"/>
+      <c r="R337" s="5"/>
     </row>
     <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I338" s="5"/>
-      <c r="Q338" s="5"/>
+      <c r="J338" s="5"/>
+      <c r="R338" s="5"/>
     </row>
     <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I339" s="5"/>
-      <c r="Q339" s="5"/>
+      <c r="J339" s="5"/>
+      <c r="R339" s="5"/>
     </row>
     <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I340" s="5"/>
-      <c r="Q340" s="5"/>
+      <c r="J340" s="5"/>
+      <c r="R340" s="5"/>
     </row>
     <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I341" s="5"/>
-      <c r="Q341" s="5"/>
+      <c r="J341" s="5"/>
+      <c r="R341" s="5"/>
     </row>
     <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I342" s="5"/>
-      <c r="Q342" s="5"/>
+      <c r="J342" s="5"/>
+      <c r="R342" s="5"/>
     </row>
     <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I343" s="5"/>
-      <c r="Q343" s="5"/>
+      <c r="J343" s="5"/>
+      <c r="R343" s="5"/>
     </row>
     <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I344" s="5"/>
-      <c r="Q344" s="5"/>
+      <c r="J344" s="5"/>
+      <c r="R344" s="5"/>
     </row>
     <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I345" s="5"/>
-      <c r="Q345" s="5"/>
+      <c r="J345" s="5"/>
+      <c r="R345" s="5"/>
     </row>
     <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I346" s="5"/>
-      <c r="Q346" s="5"/>
+      <c r="J346" s="5"/>
+      <c r="R346" s="5"/>
     </row>
     <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I347" s="5"/>
-      <c r="Q347" s="5"/>
+      <c r="J347" s="5"/>
+      <c r="R347" s="5"/>
     </row>
     <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I348" s="5"/>
-      <c r="Q348" s="5"/>
+      <c r="J348" s="5"/>
+      <c r="R348" s="5"/>
     </row>
     <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I349" s="5"/>
-      <c r="Q349" s="5"/>
+      <c r="J349" s="5"/>
+      <c r="R349" s="5"/>
     </row>
     <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I350" s="5"/>
-      <c r="Q350" s="5"/>
+      <c r="J350" s="5"/>
+      <c r="R350" s="5"/>
     </row>
     <row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I351" s="5"/>
-      <c r="Q351" s="5"/>
+      <c r="J351" s="5"/>
+      <c r="R351" s="5"/>
     </row>
     <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I352" s="5"/>
-      <c r="Q352" s="5"/>
+      <c r="J352" s="5"/>
+      <c r="R352" s="5"/>
     </row>
     <row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I353" s="5"/>
-      <c r="Q353" s="5"/>
+      <c r="J353" s="5"/>
+      <c r="R353" s="5"/>
     </row>
     <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I354" s="5"/>
-      <c r="Q354" s="5"/>
+      <c r="J354" s="5"/>
+      <c r="R354" s="5"/>
     </row>
     <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I355" s="5"/>
-      <c r="Q355" s="5"/>
+      <c r="J355" s="5"/>
+      <c r="R355" s="5"/>
     </row>
     <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I356" s="5"/>
-      <c r="Q356" s="5"/>
-    </row>
-    <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I357" s="5"/>
-      <c r="Q357" s="5"/>
-    </row>
-    <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I358" s="5"/>
-      <c r="Q358" s="5"/>
-    </row>
-    <row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I359" s="5"/>
-      <c r="Q359" s="5"/>
-    </row>
-    <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I360" s="5"/>
-      <c r="Q360" s="5"/>
-    </row>
-    <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I361" s="5"/>
-      <c r="Q361" s="5"/>
-    </row>
-    <row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I362" s="5"/>
-      <c r="Q362" s="5"/>
-    </row>
-    <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I363" s="5"/>
-      <c r="Q363" s="5"/>
-    </row>
-    <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I364" s="5"/>
-      <c r="Q364" s="5"/>
-    </row>
-    <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I365" s="5"/>
-      <c r="Q365" s="5"/>
-    </row>
-    <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I366" s="5"/>
-      <c r="Q366" s="5"/>
-    </row>
-    <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I367" s="5"/>
-      <c r="Q367" s="5"/>
-    </row>
-    <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I368" s="5"/>
-      <c r="Q368" s="5"/>
-    </row>
-    <row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I369" s="5"/>
-      <c r="Q369" s="5"/>
-    </row>
-    <row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I370" s="5"/>
-      <c r="Q370" s="5"/>
-    </row>
-    <row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I371" s="5"/>
-      <c r="Q371" s="5"/>
-    </row>
+      <c r="J356" s="5"/>
+      <c r="R356" s="5"/>
+    </row>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:R369"/>
+  <autoFilter ref="B1:S354"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3082,58 +3169,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3141,47 +3228,47 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="10"/>
       <c r="E2" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G2" s="12" t="n">
         <v>37125</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N2" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
       <c r="Q2" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R2" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3189,47 +3276,47 @@
         <v>1</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G3" s="12" t="n">
         <v>40777</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N3" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3237,47 +3324,47 @@
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G4" s="12" t="n">
         <v>33472</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N4" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
       <c r="Q4" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3285,47 +3372,47 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G5" s="12" t="n">
         <v>36760</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
       <c r="Q5" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
write error messages into import excel file (#190)
</commit_message>
<xml_diff>
--- a/tests/data/rdi_one.xlsx
+++ b/tests/data/rdi_one.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Households" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,7 +13,7 @@
     <sheet name="People" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Individuals!$A$1:$R$369</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Individuals!$B$1:$S$354</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="108">
   <si>
     <t xml:space="preserve">household_id</t>
   </si>
@@ -72,6 +72,9 @@
     <t xml:space="preserve">first_registration_date_h_c</t>
   </si>
   <si>
+    <t xml:space="preserve">head_of_household_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">MDG</t>
   </si>
   <si>
@@ -91,6 +94,9 @@
   </si>
   <si>
     <t xml:space="preserve">unicef government_partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">individual_id</t>
   </si>
   <si>
     <t xml:space="preserve">relationship_i_c</t>
@@ -540,16 +546,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>70</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>727560</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>108720</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>726840</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>108000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -562,8 +568,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16229160" y="13335120"/>
-          <a:ext cx="727560" cy="299160"/>
+          <a:off x="17254800" y="10477440"/>
+          <a:ext cx="726840" cy="298440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -577,16 +583,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>96840</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>96120</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>93960</xdr:rowOff>
+      <xdr:rowOff>93240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -599,8 +605,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9654480" y="762120"/>
-          <a:ext cx="96840" cy="93960"/>
+          <a:off x="10680120" y="762120"/>
+          <a:ext cx="96120" cy="93240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -626,9 +632,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>96840</xdr:colOff>
+      <xdr:colOff>96120</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -642,7 +648,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10336680" y="454680"/>
-          <a:ext cx="96840" cy="94320"/>
+          <a:ext cx="96120" cy="93600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -837,7 +843,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O103"/>
+  <dimension ref="A1:P103"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.33"/>
@@ -852,7 +858,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="23.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="29.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="29.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -900,6 +906,9 @@
       </c>
       <c r="O1" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -916,6 +925,7 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
@@ -926,16 +936,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>5</v>
@@ -947,323 +957,426 @@
         <v>1</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O3" s="5" t="n">
         <v>45095</v>
       </c>
+      <c r="P3" s="1" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O22" s="5"/>
+      <c r="P22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O23" s="5"/>
+      <c r="P23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O26" s="5"/>
+      <c r="P26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O27" s="5"/>
+      <c r="P27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O28" s="5"/>
+      <c r="P28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O30" s="5"/>
+      <c r="P30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O31" s="5"/>
+      <c r="P31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O32" s="5"/>
+      <c r="P32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O34" s="5"/>
+      <c r="P34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O35" s="5"/>
+      <c r="P35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O36" s="5"/>
+      <c r="P36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O37" s="5"/>
+      <c r="P37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O38" s="5"/>
+      <c r="P38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O39" s="5"/>
+      <c r="P39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O40" s="5"/>
+      <c r="P40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O41" s="5"/>
+      <c r="P41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O42" s="5"/>
+      <c r="P42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O43" s="5"/>
+      <c r="P43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O44" s="5"/>
+      <c r="P44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O45" s="5"/>
+      <c r="P45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O46" s="5"/>
+      <c r="P46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O47" s="5"/>
+      <c r="P47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O48" s="5"/>
+      <c r="P48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O49" s="5"/>
+      <c r="P49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O50" s="5"/>
+      <c r="P50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O51" s="5"/>
+      <c r="P51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O52" s="5"/>
+      <c r="P52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O53" s="5"/>
+      <c r="P53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O54" s="5"/>
+      <c r="P54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O55" s="5"/>
+      <c r="P55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O56" s="5"/>
+      <c r="P56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O57" s="5"/>
+      <c r="P57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O58" s="5"/>
+      <c r="P58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O59" s="5"/>
+      <c r="P59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O60" s="5"/>
+      <c r="P60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O61" s="5"/>
+      <c r="P61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O62" s="5"/>
+      <c r="P62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O63" s="5"/>
+      <c r="P63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O64" s="5"/>
+      <c r="P64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O65" s="5"/>
+      <c r="P65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O66" s="5"/>
+      <c r="P66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O67" s="5"/>
+      <c r="P67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O68" s="5"/>
+      <c r="P68" s="5"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O69" s="5"/>
+      <c r="P69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O70" s="5"/>
+      <c r="P70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O71" s="5"/>
+      <c r="P71" s="5"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O72" s="5"/>
+      <c r="P72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O73" s="5"/>
+      <c r="P73" s="5"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O74" s="5"/>
+      <c r="P74" s="5"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O75" s="5"/>
+      <c r="P75" s="5"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O76" s="5"/>
+      <c r="P76" s="5"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O77" s="5"/>
+      <c r="P77" s="5"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O78" s="5"/>
+      <c r="P78" s="5"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O79" s="5"/>
+      <c r="P79" s="5"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O80" s="5"/>
+      <c r="P80" s="5"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O81" s="5"/>
+      <c r="P81" s="5"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O82" s="5"/>
+      <c r="P82" s="5"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O83" s="5"/>
+      <c r="P83" s="5"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O84" s="5"/>
+      <c r="P84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O85" s="5"/>
+      <c r="P85" s="5"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O86" s="5"/>
+      <c r="P86" s="5"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O87" s="5"/>
+      <c r="P87" s="5"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O88" s="5"/>
+      <c r="P88" s="5"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O89" s="5"/>
+      <c r="P89" s="5"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O90" s="5"/>
+      <c r="P90" s="5"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O91" s="5"/>
+      <c r="P91" s="5"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O92" s="5"/>
+      <c r="P92" s="5"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O93" s="5"/>
+      <c r="P93" s="5"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O94" s="5"/>
+      <c r="P94" s="5"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O95" s="5"/>
+      <c r="P95" s="5"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O96" s="5"/>
+      <c r="P96" s="5"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O97" s="5"/>
+      <c r="P97" s="5"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O98" s="5"/>
+      <c r="P98" s="5"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O99" s="5"/>
+      <c r="P99" s="5"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O100" s="5"/>
+      <c r="P100" s="5"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O101" s="5"/>
+      <c r="P101" s="5"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O102" s="5"/>
+      <c r="P102" s="5"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O103" s="5"/>
+      <c r="P103" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1281,86 +1394,89 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R371"/>
+  <dimension ref="A1:S1048576"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="19.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="19.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="11.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="35.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="15.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="13.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="17.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="21.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="19.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="18.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="19.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="11.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="C1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -1378,1672 +1494,1643 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>39</v>
+      <c r="B3" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="G3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="5" t="n">
         <v>28558</v>
       </c>
-      <c r="J3" s="4" t="b">
+      <c r="K3" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>15</v>
+      <c r="L3" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="O3" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="P3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q3" s="5" t="n">
+      <c r="R3" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R3" s="6" t="s">
-        <v>47</v>
+      <c r="S3" s="6" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I4" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J4" s="5" t="n">
         <v>24971</v>
       </c>
-      <c r="J4" s="4" t="b">
+      <c r="K4" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="Q4" s="5" t="n">
+      <c r="R4" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R4" s="6" t="s">
-        <v>52</v>
+      <c r="S4" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I5" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J5" s="5" t="n">
         <v>24092</v>
       </c>
-      <c r="J5" s="4" t="b">
+      <c r="K5" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K5" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="P5" s="1" t="n">
+      <c r="L5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="Q5" s="5" t="n">
+      <c r="R5" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R5" s="6" t="s">
-        <v>52</v>
+      <c r="S5" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="C6" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="I6" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="5" t="n">
         <v>43298</v>
       </c>
-      <c r="J6" s="4" t="b">
+      <c r="K6" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q6" s="5" t="n">
+      <c r="L6" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="R6" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R6" s="6" t="s">
-        <v>52</v>
+      <c r="S6" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I7" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J7" s="5" t="n">
         <v>34615</v>
       </c>
-      <c r="J7" s="4" t="b">
+      <c r="K7" s="4" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="Q7" s="5" t="n">
+      <c r="R7" s="5" t="n">
         <v>45095</v>
       </c>
-      <c r="R7" s="6" t="s">
-        <v>52</v>
+      <c r="S7" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I8" s="5"/>
-      <c r="Q8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="R8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I9" s="5"/>
-      <c r="Q9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="R9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I10" s="5"/>
-      <c r="Q10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="R10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I11" s="5"/>
-      <c r="Q11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="R11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I12" s="5"/>
-      <c r="Q12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="R12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I13" s="5"/>
-      <c r="Q13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="R13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I14" s="5"/>
-      <c r="Q14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="R14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I15" s="5"/>
-      <c r="Q15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="R15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I16" s="5"/>
-      <c r="Q16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="R16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I17" s="5"/>
-      <c r="Q17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="R17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I18" s="5"/>
-      <c r="Q18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="R18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I19" s="5"/>
-      <c r="Q19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="R19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I20" s="5"/>
-      <c r="Q20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="R20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I21" s="5"/>
-      <c r="Q21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="R21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I22" s="5"/>
-      <c r="Q22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="R22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I23" s="5"/>
-      <c r="Q23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="R23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I24" s="5"/>
-      <c r="Q24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="R24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I25" s="5"/>
-      <c r="Q25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="R25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I26" s="5"/>
-      <c r="Q26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="R26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I27" s="5"/>
-      <c r="Q27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="R27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I28" s="5"/>
-      <c r="Q28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="R28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I29" s="5"/>
-      <c r="Q29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="R29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I30" s="5"/>
-      <c r="Q30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="R30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I31" s="5"/>
-      <c r="Q31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="R31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I32" s="5"/>
-      <c r="Q32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="R32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I33" s="5"/>
-      <c r="Q33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="R33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I34" s="5"/>
-      <c r="Q34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="R34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I35" s="5"/>
-      <c r="Q35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="R35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I36" s="5"/>
-      <c r="Q36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="R36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I37" s="5"/>
-      <c r="Q37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="R37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I38" s="5"/>
-      <c r="Q38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="R38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I39" s="5"/>
-      <c r="Q39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="R39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I40" s="5"/>
-      <c r="Q40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="R40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I41" s="5"/>
-      <c r="Q41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="R41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I42" s="5"/>
-      <c r="Q42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="R42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I43" s="5"/>
-      <c r="Q43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="R43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I44" s="5"/>
-      <c r="Q44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="R44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I45" s="5"/>
-      <c r="Q45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="R45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I46" s="5"/>
-      <c r="Q46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="R46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I47" s="5"/>
-      <c r="Q47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="R47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I48" s="5"/>
-      <c r="Q48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="R48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I49" s="5"/>
-      <c r="Q49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="R49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I50" s="5"/>
-      <c r="Q50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="R50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I51" s="5"/>
-      <c r="Q51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="R51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I52" s="5"/>
-      <c r="Q52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="R52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I53" s="5"/>
-      <c r="Q53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="R53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I54" s="5"/>
-      <c r="Q54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="R54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I55" s="5"/>
-      <c r="Q55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="R55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I56" s="5"/>
-      <c r="Q56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="R56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I57" s="5"/>
-      <c r="Q57" s="5"/>
+      <c r="J57" s="5"/>
+      <c r="R57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I58" s="5"/>
-      <c r="Q58" s="5"/>
+      <c r="J58" s="5"/>
+      <c r="R58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I59" s="5"/>
-      <c r="Q59" s="5"/>
+      <c r="J59" s="5"/>
+      <c r="R59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I60" s="5"/>
-      <c r="Q60" s="5"/>
+      <c r="J60" s="5"/>
+      <c r="R60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I61" s="5"/>
-      <c r="Q61" s="5"/>
+      <c r="J61" s="5"/>
+      <c r="R61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I62" s="5"/>
-      <c r="Q62" s="5"/>
+      <c r="J62" s="5"/>
+      <c r="R62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I63" s="5"/>
-      <c r="Q63" s="5"/>
+      <c r="J63" s="5"/>
+      <c r="R63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I64" s="5"/>
-      <c r="Q64" s="5"/>
+      <c r="J64" s="5"/>
+      <c r="R64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I65" s="5"/>
-      <c r="Q65" s="5"/>
+      <c r="J65" s="5"/>
+      <c r="R65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I66" s="5"/>
-      <c r="Q66" s="5"/>
+      <c r="J66" s="5"/>
+      <c r="R66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I67" s="5"/>
-      <c r="Q67" s="5"/>
+      <c r="J67" s="5"/>
+      <c r="R67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I68" s="5"/>
-      <c r="Q68" s="5"/>
+      <c r="J68" s="5"/>
+      <c r="R68" s="5"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I69" s="5"/>
-      <c r="Q69" s="5"/>
+      <c r="J69" s="5"/>
+      <c r="R69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I70" s="5"/>
-      <c r="Q70" s="5"/>
+      <c r="J70" s="5"/>
+      <c r="R70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I71" s="5"/>
-      <c r="Q71" s="5"/>
+      <c r="J71" s="5"/>
+      <c r="R71" s="5"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I72" s="5"/>
-      <c r="Q72" s="5"/>
+      <c r="J72" s="5"/>
+      <c r="R72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I73" s="5"/>
-      <c r="Q73" s="5"/>
+      <c r="J73" s="5"/>
+      <c r="R73" s="5"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I74" s="5"/>
-      <c r="Q74" s="5"/>
+      <c r="J74" s="5"/>
+      <c r="R74" s="5"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I75" s="5"/>
-      <c r="Q75" s="5"/>
+      <c r="J75" s="5"/>
+      <c r="R75" s="5"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I76" s="5"/>
-      <c r="Q76" s="5"/>
+      <c r="J76" s="5"/>
+      <c r="R76" s="5"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I77" s="5"/>
-      <c r="Q77" s="5"/>
+      <c r="J77" s="5"/>
+      <c r="R77" s="5"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I78" s="5"/>
-      <c r="Q78" s="5"/>
+      <c r="J78" s="5"/>
+      <c r="R78" s="5"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I79" s="5"/>
-      <c r="Q79" s="5"/>
+      <c r="J79" s="5"/>
+      <c r="R79" s="5"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I80" s="5"/>
-      <c r="Q80" s="5"/>
+      <c r="J80" s="5"/>
+      <c r="R80" s="5"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I81" s="5"/>
-      <c r="Q81" s="5"/>
+      <c r="J81" s="5"/>
+      <c r="R81" s="5"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I82" s="5"/>
-      <c r="Q82" s="5"/>
+      <c r="J82" s="5"/>
+      <c r="R82" s="5"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I83" s="5"/>
-      <c r="Q83" s="5"/>
+      <c r="J83" s="5"/>
+      <c r="R83" s="5"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I84" s="5"/>
-      <c r="Q84" s="5"/>
+      <c r="J84" s="5"/>
+      <c r="R84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I85" s="5"/>
-      <c r="Q85" s="5"/>
+      <c r="J85" s="5"/>
+      <c r="R85" s="5"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I86" s="5"/>
-      <c r="Q86" s="5"/>
+      <c r="J86" s="5"/>
+      <c r="R86" s="5"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I87" s="5"/>
-      <c r="Q87" s="5"/>
+      <c r="J87" s="5"/>
+      <c r="R87" s="5"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I88" s="5"/>
-      <c r="Q88" s="5"/>
+      <c r="J88" s="5"/>
+      <c r="R88" s="5"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I89" s="5"/>
-      <c r="Q89" s="5"/>
+      <c r="J89" s="5"/>
+      <c r="R89" s="5"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I90" s="5"/>
-      <c r="Q90" s="5"/>
+      <c r="J90" s="5"/>
+      <c r="R90" s="5"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I91" s="5"/>
-      <c r="Q91" s="5"/>
+      <c r="J91" s="5"/>
+      <c r="R91" s="5"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I92" s="5"/>
-      <c r="Q92" s="5"/>
+      <c r="J92" s="5"/>
+      <c r="R92" s="5"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I93" s="5"/>
-      <c r="Q93" s="5"/>
+      <c r="J93" s="5"/>
+      <c r="R93" s="5"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I94" s="5"/>
-      <c r="Q94" s="5"/>
+      <c r="J94" s="5"/>
+      <c r="R94" s="5"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I95" s="5"/>
-      <c r="Q95" s="5"/>
+      <c r="J95" s="5"/>
+      <c r="R95" s="5"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I96" s="5"/>
-      <c r="Q96" s="5"/>
+      <c r="J96" s="5"/>
+      <c r="R96" s="5"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I97" s="5"/>
-      <c r="Q97" s="5"/>
+      <c r="J97" s="5"/>
+      <c r="R97" s="5"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I98" s="5"/>
-      <c r="Q98" s="5"/>
+      <c r="J98" s="5"/>
+      <c r="R98" s="5"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I99" s="5"/>
-      <c r="Q99" s="5"/>
+      <c r="J99" s="5"/>
+      <c r="R99" s="5"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I100" s="5"/>
-      <c r="Q100" s="5"/>
+      <c r="J100" s="5"/>
+      <c r="R100" s="5"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I101" s="5"/>
-      <c r="Q101" s="5"/>
+      <c r="J101" s="5"/>
+      <c r="R101" s="5"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I102" s="5"/>
-      <c r="Q102" s="5"/>
+      <c r="J102" s="5"/>
+      <c r="R102" s="5"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I103" s="5"/>
-      <c r="Q103" s="5"/>
+      <c r="J103" s="5"/>
+      <c r="R103" s="5"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I104" s="5"/>
-      <c r="Q104" s="5"/>
+      <c r="J104" s="5"/>
+      <c r="R104" s="5"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I105" s="5"/>
-      <c r="Q105" s="5"/>
+      <c r="J105" s="5"/>
+      <c r="R105" s="5"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I106" s="5"/>
-      <c r="Q106" s="5"/>
+      <c r="J106" s="5"/>
+      <c r="R106" s="5"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I107" s="5"/>
-      <c r="Q107" s="5"/>
+      <c r="J107" s="5"/>
+      <c r="R107" s="5"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I108" s="5"/>
-      <c r="Q108" s="5"/>
+      <c r="J108" s="5"/>
+      <c r="R108" s="5"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I109" s="5"/>
-      <c r="Q109" s="5"/>
+      <c r="J109" s="5"/>
+      <c r="R109" s="5"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I110" s="5"/>
-      <c r="Q110" s="5"/>
+      <c r="J110" s="5"/>
+      <c r="R110" s="5"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I111" s="5"/>
-      <c r="Q111" s="5"/>
+      <c r="J111" s="5"/>
+      <c r="R111" s="5"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I112" s="5"/>
-      <c r="Q112" s="5"/>
+      <c r="J112" s="5"/>
+      <c r="R112" s="5"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I113" s="5"/>
-      <c r="Q113" s="5"/>
+      <c r="J113" s="5"/>
+      <c r="R113" s="5"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I114" s="5"/>
-      <c r="Q114" s="5"/>
+      <c r="J114" s="5"/>
+      <c r="R114" s="5"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I115" s="5"/>
-      <c r="Q115" s="5"/>
+      <c r="J115" s="5"/>
+      <c r="R115" s="5"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I116" s="5"/>
-      <c r="Q116" s="5"/>
+      <c r="J116" s="5"/>
+      <c r="R116" s="5"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I117" s="5"/>
-      <c r="Q117" s="5"/>
+      <c r="J117" s="5"/>
+      <c r="R117" s="5"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I118" s="5"/>
-      <c r="Q118" s="5"/>
+      <c r="J118" s="5"/>
+      <c r="R118" s="5"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I119" s="5"/>
-      <c r="Q119" s="5"/>
+      <c r="J119" s="5"/>
+      <c r="R119" s="5"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I120" s="5"/>
-      <c r="Q120" s="5"/>
+      <c r="J120" s="5"/>
+      <c r="R120" s="5"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I121" s="5"/>
-      <c r="Q121" s="5"/>
+      <c r="J121" s="5"/>
+      <c r="R121" s="5"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I122" s="5"/>
-      <c r="Q122" s="5"/>
+      <c r="J122" s="5"/>
+      <c r="R122" s="5"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I123" s="5"/>
-      <c r="Q123" s="5"/>
+      <c r="J123" s="5"/>
+      <c r="R123" s="5"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I124" s="5"/>
-      <c r="Q124" s="5"/>
+      <c r="J124" s="5"/>
+      <c r="R124" s="5"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I125" s="5"/>
-      <c r="Q125" s="5"/>
+      <c r="J125" s="5"/>
+      <c r="R125" s="5"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I126" s="5"/>
-      <c r="Q126" s="5"/>
+      <c r="J126" s="5"/>
+      <c r="R126" s="5"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I127" s="5"/>
-      <c r="Q127" s="5"/>
+      <c r="J127" s="5"/>
+      <c r="R127" s="5"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I128" s="5"/>
-      <c r="Q128" s="5"/>
+      <c r="J128" s="5"/>
+      <c r="R128" s="5"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I129" s="5"/>
-      <c r="Q129" s="5"/>
+      <c r="J129" s="5"/>
+      <c r="R129" s="5"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I130" s="5"/>
-      <c r="Q130" s="5"/>
+      <c r="J130" s="5"/>
+      <c r="R130" s="5"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I131" s="5"/>
-      <c r="Q131" s="5"/>
+      <c r="J131" s="5"/>
+      <c r="R131" s="5"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I132" s="5"/>
-      <c r="Q132" s="5"/>
+      <c r="J132" s="5"/>
+      <c r="R132" s="5"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I133" s="5"/>
-      <c r="Q133" s="5"/>
+      <c r="J133" s="5"/>
+      <c r="R133" s="5"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I134" s="5"/>
-      <c r="Q134" s="5"/>
+      <c r="J134" s="5"/>
+      <c r="R134" s="5"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I135" s="5"/>
-      <c r="Q135" s="5"/>
+      <c r="J135" s="5"/>
+      <c r="R135" s="5"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I136" s="5"/>
-      <c r="Q136" s="5"/>
+      <c r="J136" s="5"/>
+      <c r="R136" s="5"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I137" s="5"/>
-      <c r="Q137" s="5"/>
+      <c r="J137" s="5"/>
+      <c r="R137" s="5"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I138" s="5"/>
-      <c r="Q138" s="5"/>
+      <c r="J138" s="5"/>
+      <c r="R138" s="5"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I139" s="5"/>
-      <c r="Q139" s="5"/>
+      <c r="J139" s="5"/>
+      <c r="R139" s="5"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I140" s="5"/>
-      <c r="Q140" s="5"/>
+      <c r="J140" s="5"/>
+      <c r="R140" s="5"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I141" s="5"/>
-      <c r="Q141" s="5"/>
+      <c r="J141" s="5"/>
+      <c r="R141" s="5"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I142" s="5"/>
-      <c r="Q142" s="5"/>
+      <c r="J142" s="5"/>
+      <c r="R142" s="5"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I143" s="5"/>
-      <c r="Q143" s="5"/>
+      <c r="J143" s="5"/>
+      <c r="R143" s="5"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I144" s="5"/>
-      <c r="Q144" s="5"/>
+      <c r="J144" s="5"/>
+      <c r="R144" s="5"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I145" s="5"/>
-      <c r="Q145" s="5"/>
+      <c r="J145" s="5"/>
+      <c r="R145" s="5"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I146" s="5"/>
-      <c r="Q146" s="5"/>
+      <c r="J146" s="5"/>
+      <c r="R146" s="5"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I147" s="5"/>
-      <c r="Q147" s="5"/>
+      <c r="J147" s="5"/>
+      <c r="R147" s="5"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I148" s="5"/>
-      <c r="Q148" s="5"/>
+      <c r="J148" s="5"/>
+      <c r="R148" s="5"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I149" s="5"/>
-      <c r="Q149" s="5"/>
+      <c r="J149" s="5"/>
+      <c r="R149" s="5"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I150" s="5"/>
-      <c r="Q150" s="5"/>
+      <c r="J150" s="5"/>
+      <c r="R150" s="5"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I151" s="5"/>
-      <c r="Q151" s="5"/>
+      <c r="J151" s="5"/>
+      <c r="R151" s="5"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I152" s="5"/>
-      <c r="Q152" s="5"/>
+      <c r="J152" s="5"/>
+      <c r="R152" s="5"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I153" s="5"/>
-      <c r="Q153" s="5"/>
+      <c r="J153" s="5"/>
+      <c r="R153" s="5"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I154" s="5"/>
-      <c r="Q154" s="5"/>
+      <c r="J154" s="5"/>
+      <c r="R154" s="5"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I155" s="5"/>
-      <c r="Q155" s="5"/>
+      <c r="J155" s="5"/>
+      <c r="R155" s="5"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I156" s="5"/>
-      <c r="Q156" s="5"/>
+      <c r="J156" s="5"/>
+      <c r="R156" s="5"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I157" s="5"/>
-      <c r="Q157" s="5"/>
+      <c r="J157" s="5"/>
+      <c r="R157" s="5"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I158" s="5"/>
-      <c r="Q158" s="5"/>
+      <c r="J158" s="5"/>
+      <c r="R158" s="5"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I159" s="5"/>
-      <c r="Q159" s="5"/>
+      <c r="J159" s="5"/>
+      <c r="R159" s="5"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I160" s="5"/>
-      <c r="Q160" s="5"/>
+      <c r="J160" s="5"/>
+      <c r="R160" s="5"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I161" s="5"/>
-      <c r="Q161" s="5"/>
+      <c r="J161" s="5"/>
+      <c r="R161" s="5"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I162" s="5"/>
-      <c r="Q162" s="5"/>
+      <c r="J162" s="5"/>
+      <c r="R162" s="5"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I163" s="5"/>
-      <c r="Q163" s="5"/>
+      <c r="J163" s="5"/>
+      <c r="R163" s="5"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I164" s="5"/>
-      <c r="Q164" s="5"/>
+      <c r="J164" s="5"/>
+      <c r="R164" s="5"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I165" s="5"/>
-      <c r="Q165" s="5"/>
+      <c r="J165" s="5"/>
+      <c r="R165" s="5"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I166" s="5"/>
-      <c r="Q166" s="5"/>
+      <c r="J166" s="5"/>
+      <c r="R166" s="5"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I167" s="5"/>
-      <c r="Q167" s="5"/>
+      <c r="J167" s="5"/>
+      <c r="R167" s="5"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I168" s="5"/>
-      <c r="Q168" s="5"/>
+      <c r="J168" s="5"/>
+      <c r="R168" s="5"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I169" s="5"/>
-      <c r="Q169" s="5"/>
+      <c r="J169" s="5"/>
+      <c r="R169" s="5"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I170" s="5"/>
-      <c r="Q170" s="5"/>
+      <c r="J170" s="5"/>
+      <c r="R170" s="5"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I171" s="5"/>
-      <c r="Q171" s="5"/>
+      <c r="J171" s="5"/>
+      <c r="R171" s="5"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I172" s="5"/>
-      <c r="Q172" s="5"/>
+      <c r="J172" s="5"/>
+      <c r="R172" s="5"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I173" s="5"/>
-      <c r="Q173" s="5"/>
+      <c r="J173" s="5"/>
+      <c r="R173" s="5"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I174" s="5"/>
-      <c r="Q174" s="5"/>
+      <c r="J174" s="5"/>
+      <c r="R174" s="5"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I175" s="5"/>
-      <c r="Q175" s="5"/>
+      <c r="J175" s="5"/>
+      <c r="R175" s="5"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I176" s="5"/>
-      <c r="Q176" s="5"/>
+      <c r="J176" s="5"/>
+      <c r="R176" s="5"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I177" s="5"/>
-      <c r="Q177" s="5"/>
+      <c r="J177" s="5"/>
+      <c r="R177" s="5"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I178" s="5"/>
-      <c r="Q178" s="5"/>
+      <c r="J178" s="5"/>
+      <c r="R178" s="5"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I179" s="5"/>
-      <c r="Q179" s="5"/>
+      <c r="J179" s="5"/>
+      <c r="R179" s="5"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I180" s="5"/>
-      <c r="Q180" s="5"/>
+      <c r="J180" s="5"/>
+      <c r="R180" s="5"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I181" s="5"/>
-      <c r="Q181" s="5"/>
+      <c r="J181" s="5"/>
+      <c r="R181" s="5"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I182" s="5"/>
-      <c r="Q182" s="5"/>
+      <c r="J182" s="5"/>
+      <c r="R182" s="5"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I183" s="5"/>
-      <c r="Q183" s="5"/>
+      <c r="J183" s="5"/>
+      <c r="R183" s="5"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I184" s="5"/>
-      <c r="Q184" s="5"/>
+      <c r="J184" s="5"/>
+      <c r="R184" s="5"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I185" s="5"/>
-      <c r="Q185" s="5"/>
+      <c r="J185" s="5"/>
+      <c r="R185" s="5"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I186" s="5"/>
-      <c r="Q186" s="5"/>
+      <c r="J186" s="5"/>
+      <c r="R186" s="5"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I187" s="5"/>
-      <c r="Q187" s="5"/>
+      <c r="J187" s="5"/>
+      <c r="R187" s="5"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I188" s="5"/>
-      <c r="Q188" s="5"/>
+      <c r="J188" s="5"/>
+      <c r="R188" s="5"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I189" s="5"/>
-      <c r="Q189" s="5"/>
+      <c r="J189" s="5"/>
+      <c r="R189" s="5"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I190" s="5"/>
-      <c r="Q190" s="5"/>
+      <c r="J190" s="5"/>
+      <c r="R190" s="5"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I191" s="5"/>
-      <c r="Q191" s="5"/>
+      <c r="J191" s="5"/>
+      <c r="R191" s="5"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I192" s="5"/>
-      <c r="Q192" s="5"/>
+      <c r="J192" s="5"/>
+      <c r="R192" s="5"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I193" s="5"/>
-      <c r="Q193" s="5"/>
+      <c r="J193" s="5"/>
+      <c r="R193" s="5"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I194" s="5"/>
-      <c r="Q194" s="5"/>
+      <c r="J194" s="5"/>
+      <c r="R194" s="5"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I195" s="5"/>
-      <c r="Q195" s="5"/>
+      <c r="J195" s="5"/>
+      <c r="R195" s="5"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I196" s="5"/>
-      <c r="Q196" s="5"/>
+      <c r="J196" s="5"/>
+      <c r="R196" s="5"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I197" s="5"/>
-      <c r="Q197" s="5"/>
+      <c r="J197" s="5"/>
+      <c r="R197" s="5"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I198" s="5"/>
-      <c r="Q198" s="5"/>
+      <c r="J198" s="5"/>
+      <c r="R198" s="5"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I199" s="5"/>
-      <c r="Q199" s="5"/>
+      <c r="J199" s="5"/>
+      <c r="R199" s="5"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I200" s="5"/>
-      <c r="Q200" s="5"/>
+      <c r="J200" s="5"/>
+      <c r="R200" s="5"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I201" s="5"/>
-      <c r="Q201" s="5"/>
+      <c r="J201" s="5"/>
+      <c r="R201" s="5"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I202" s="5"/>
-      <c r="Q202" s="5"/>
+      <c r="J202" s="5"/>
+      <c r="R202" s="5"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I203" s="5"/>
-      <c r="Q203" s="5"/>
+      <c r="J203" s="5"/>
+      <c r="R203" s="5"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I204" s="5"/>
-      <c r="Q204" s="5"/>
+      <c r="J204" s="5"/>
+      <c r="R204" s="5"/>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I205" s="5"/>
-      <c r="Q205" s="5"/>
+      <c r="J205" s="5"/>
+      <c r="R205" s="5"/>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I206" s="5"/>
-      <c r="Q206" s="5"/>
+      <c r="J206" s="5"/>
+      <c r="R206" s="5"/>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I207" s="5"/>
-      <c r="Q207" s="5"/>
+      <c r="J207" s="5"/>
+      <c r="R207" s="5"/>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I208" s="5"/>
-      <c r="Q208" s="5"/>
+      <c r="J208" s="5"/>
+      <c r="R208" s="5"/>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I209" s="5"/>
-      <c r="Q209" s="5"/>
+      <c r="J209" s="5"/>
+      <c r="R209" s="5"/>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I210" s="5"/>
-      <c r="Q210" s="5"/>
+      <c r="J210" s="5"/>
+      <c r="R210" s="5"/>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I211" s="5"/>
-      <c r="Q211" s="5"/>
+      <c r="J211" s="5"/>
+      <c r="R211" s="5"/>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I212" s="5"/>
-      <c r="Q212" s="5"/>
+      <c r="J212" s="5"/>
+      <c r="R212" s="5"/>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I213" s="5"/>
-      <c r="Q213" s="5"/>
+      <c r="J213" s="5"/>
+      <c r="R213" s="5"/>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I214" s="5"/>
-      <c r="Q214" s="5"/>
+      <c r="J214" s="5"/>
+      <c r="R214" s="5"/>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I215" s="5"/>
-      <c r="Q215" s="5"/>
+      <c r="J215" s="5"/>
+      <c r="R215" s="5"/>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I216" s="5"/>
-      <c r="Q216" s="5"/>
+      <c r="J216" s="5"/>
+      <c r="R216" s="5"/>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I217" s="5"/>
-      <c r="Q217" s="5"/>
+      <c r="J217" s="5"/>
+      <c r="R217" s="5"/>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I218" s="5"/>
-      <c r="Q218" s="5"/>
+      <c r="J218" s="5"/>
+      <c r="R218" s="5"/>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I219" s="5"/>
-      <c r="Q219" s="5"/>
+      <c r="J219" s="5"/>
+      <c r="R219" s="5"/>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I220" s="5"/>
-      <c r="Q220" s="5"/>
+      <c r="J220" s="5"/>
+      <c r="R220" s="5"/>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I221" s="5"/>
-      <c r="Q221" s="5"/>
+      <c r="J221" s="5"/>
+      <c r="R221" s="5"/>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I222" s="5"/>
-      <c r="Q222" s="5"/>
+      <c r="J222" s="5"/>
+      <c r="R222" s="5"/>
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I223" s="5"/>
-      <c r="Q223" s="5"/>
+      <c r="J223" s="5"/>
+      <c r="R223" s="5"/>
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I224" s="5"/>
-      <c r="Q224" s="5"/>
+      <c r="J224" s="5"/>
+      <c r="R224" s="5"/>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I225" s="5"/>
-      <c r="Q225" s="5"/>
+      <c r="J225" s="5"/>
+      <c r="R225" s="5"/>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I226" s="5"/>
-      <c r="Q226" s="5"/>
+      <c r="J226" s="5"/>
+      <c r="R226" s="5"/>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I227" s="5"/>
-      <c r="Q227" s="5"/>
+      <c r="J227" s="5"/>
+      <c r="R227" s="5"/>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I228" s="5"/>
-      <c r="Q228" s="5"/>
+      <c r="J228" s="5"/>
+      <c r="R228" s="5"/>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I229" s="5"/>
-      <c r="Q229" s="5"/>
+      <c r="J229" s="5"/>
+      <c r="R229" s="5"/>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I230" s="5"/>
-      <c r="Q230" s="5"/>
+      <c r="J230" s="5"/>
+      <c r="R230" s="5"/>
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I231" s="5"/>
-      <c r="Q231" s="5"/>
+      <c r="J231" s="5"/>
+      <c r="R231" s="5"/>
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I232" s="5"/>
-      <c r="Q232" s="5"/>
+      <c r="J232" s="5"/>
+      <c r="R232" s="5"/>
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I233" s="5"/>
-      <c r="Q233" s="5"/>
+      <c r="J233" s="5"/>
+      <c r="R233" s="5"/>
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I234" s="5"/>
-      <c r="Q234" s="5"/>
+      <c r="J234" s="5"/>
+      <c r="R234" s="5"/>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I235" s="5"/>
-      <c r="Q235" s="5"/>
+      <c r="J235" s="5"/>
+      <c r="R235" s="5"/>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I236" s="5"/>
-      <c r="Q236" s="5"/>
+      <c r="J236" s="5"/>
+      <c r="R236" s="5"/>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I237" s="5"/>
-      <c r="Q237" s="5"/>
+      <c r="J237" s="5"/>
+      <c r="R237" s="5"/>
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I238" s="5"/>
-      <c r="Q238" s="5"/>
+      <c r="J238" s="5"/>
+      <c r="R238" s="5"/>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I239" s="5"/>
-      <c r="Q239" s="5"/>
+      <c r="J239" s="5"/>
+      <c r="R239" s="5"/>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I240" s="5"/>
-      <c r="Q240" s="5"/>
+      <c r="J240" s="5"/>
+      <c r="R240" s="5"/>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I241" s="5"/>
-      <c r="Q241" s="5"/>
+      <c r="J241" s="5"/>
+      <c r="R241" s="5"/>
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I242" s="5"/>
-      <c r="Q242" s="5"/>
+      <c r="J242" s="5"/>
+      <c r="R242" s="5"/>
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I243" s="5"/>
-      <c r="Q243" s="5"/>
+      <c r="J243" s="5"/>
+      <c r="R243" s="5"/>
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I244" s="5"/>
-      <c r="Q244" s="5"/>
+      <c r="J244" s="5"/>
+      <c r="R244" s="5"/>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I245" s="5"/>
-      <c r="Q245" s="5"/>
+      <c r="J245" s="5"/>
+      <c r="R245" s="5"/>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I246" s="5"/>
-      <c r="Q246" s="5"/>
+      <c r="J246" s="5"/>
+      <c r="R246" s="5"/>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I247" s="5"/>
-      <c r="Q247" s="5"/>
+      <c r="J247" s="5"/>
+      <c r="R247" s="5"/>
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I248" s="5"/>
-      <c r="Q248" s="5"/>
+      <c r="J248" s="5"/>
+      <c r="R248" s="5"/>
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I249" s="5"/>
-      <c r="Q249" s="5"/>
+      <c r="J249" s="5"/>
+      <c r="R249" s="5"/>
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I250" s="5"/>
-      <c r="Q250" s="5"/>
+      <c r="J250" s="5"/>
+      <c r="R250" s="5"/>
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I251" s="5"/>
-      <c r="Q251" s="5"/>
+      <c r="J251" s="5"/>
+      <c r="R251" s="5"/>
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I252" s="5"/>
-      <c r="Q252" s="5"/>
+      <c r="J252" s="5"/>
+      <c r="R252" s="5"/>
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I253" s="5"/>
-      <c r="Q253" s="5"/>
+      <c r="J253" s="5"/>
+      <c r="R253" s="5"/>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I254" s="5"/>
-      <c r="Q254" s="5"/>
+      <c r="J254" s="5"/>
+      <c r="R254" s="5"/>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I255" s="5"/>
-      <c r="Q255" s="5"/>
+      <c r="J255" s="5"/>
+      <c r="R255" s="5"/>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I256" s="5"/>
-      <c r="Q256" s="5"/>
+      <c r="J256" s="5"/>
+      <c r="R256" s="5"/>
     </row>
     <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I257" s="5"/>
-      <c r="Q257" s="5"/>
+      <c r="J257" s="5"/>
+      <c r="R257" s="5"/>
     </row>
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I258" s="5"/>
-      <c r="Q258" s="5"/>
+      <c r="J258" s="5"/>
+      <c r="R258" s="5"/>
     </row>
     <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I259" s="5"/>
-      <c r="Q259" s="5"/>
+      <c r="J259" s="5"/>
+      <c r="R259" s="5"/>
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I260" s="5"/>
-      <c r="Q260" s="5"/>
+      <c r="J260" s="5"/>
+      <c r="R260" s="5"/>
     </row>
     <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I261" s="5"/>
-      <c r="Q261" s="5"/>
+      <c r="J261" s="5"/>
+      <c r="R261" s="5"/>
     </row>
     <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I262" s="5"/>
-      <c r="Q262" s="5"/>
+      <c r="J262" s="5"/>
+      <c r="R262" s="5"/>
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I263" s="5"/>
-      <c r="Q263" s="5"/>
+      <c r="J263" s="5"/>
+      <c r="R263" s="5"/>
     </row>
     <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I264" s="5"/>
-      <c r="Q264" s="5"/>
+      <c r="J264" s="5"/>
+      <c r="R264" s="5"/>
     </row>
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I265" s="5"/>
-      <c r="Q265" s="5"/>
+      <c r="J265" s="5"/>
+      <c r="R265" s="5"/>
     </row>
     <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I266" s="5"/>
-      <c r="Q266" s="5"/>
+      <c r="J266" s="5"/>
+      <c r="R266" s="5"/>
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I267" s="5"/>
-      <c r="Q267" s="5"/>
+      <c r="J267" s="5"/>
+      <c r="R267" s="5"/>
     </row>
     <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I268" s="5"/>
-      <c r="Q268" s="5"/>
+      <c r="J268" s="5"/>
+      <c r="R268" s="5"/>
     </row>
     <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I269" s="5"/>
-      <c r="Q269" s="5"/>
+      <c r="J269" s="5"/>
+      <c r="R269" s="5"/>
     </row>
     <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I270" s="5"/>
-      <c r="Q270" s="5"/>
+      <c r="J270" s="5"/>
+      <c r="R270" s="5"/>
     </row>
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I271" s="5"/>
-      <c r="Q271" s="5"/>
+      <c r="J271" s="5"/>
+      <c r="R271" s="5"/>
     </row>
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I272" s="5"/>
-      <c r="Q272" s="5"/>
+      <c r="J272" s="5"/>
+      <c r="R272" s="5"/>
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I273" s="5"/>
-      <c r="Q273" s="5"/>
+      <c r="J273" s="5"/>
+      <c r="R273" s="5"/>
     </row>
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I274" s="5"/>
-      <c r="Q274" s="5"/>
+      <c r="J274" s="5"/>
+      <c r="R274" s="5"/>
     </row>
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I275" s="5"/>
-      <c r="Q275" s="5"/>
+      <c r="J275" s="5"/>
+      <c r="R275" s="5"/>
     </row>
     <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I276" s="5"/>
-      <c r="Q276" s="5"/>
+      <c r="J276" s="5"/>
+      <c r="R276" s="5"/>
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I277" s="5"/>
-      <c r="Q277" s="5"/>
+      <c r="J277" s="5"/>
+      <c r="R277" s="5"/>
     </row>
     <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I278" s="5"/>
-      <c r="Q278" s="5"/>
+      <c r="J278" s="5"/>
+      <c r="R278" s="5"/>
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I279" s="5"/>
-      <c r="Q279" s="5"/>
+      <c r="J279" s="5"/>
+      <c r="R279" s="5"/>
     </row>
     <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I280" s="5"/>
-      <c r="Q280" s="5"/>
+      <c r="J280" s="5"/>
+      <c r="R280" s="5"/>
     </row>
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I281" s="5"/>
-      <c r="Q281" s="5"/>
+      <c r="J281" s="5"/>
+      <c r="R281" s="5"/>
     </row>
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I282" s="5"/>
-      <c r="Q282" s="5"/>
+      <c r="J282" s="5"/>
+      <c r="R282" s="5"/>
     </row>
     <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I283" s="5"/>
-      <c r="Q283" s="5"/>
+      <c r="J283" s="5"/>
+      <c r="R283" s="5"/>
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I284" s="5"/>
-      <c r="Q284" s="5"/>
+      <c r="J284" s="5"/>
+      <c r="R284" s="5"/>
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I285" s="5"/>
-      <c r="Q285" s="5"/>
+      <c r="J285" s="5"/>
+      <c r="R285" s="5"/>
     </row>
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I286" s="5"/>
-      <c r="Q286" s="5"/>
+      <c r="J286" s="5"/>
+      <c r="R286" s="5"/>
     </row>
     <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I287" s="5"/>
-      <c r="Q287" s="5"/>
+      <c r="J287" s="5"/>
+      <c r="R287" s="5"/>
     </row>
     <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I288" s="5"/>
-      <c r="Q288" s="5"/>
+      <c r="J288" s="5"/>
+      <c r="R288" s="5"/>
     </row>
     <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I289" s="5"/>
-      <c r="Q289" s="5"/>
+      <c r="J289" s="5"/>
+      <c r="R289" s="5"/>
     </row>
     <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I290" s="5"/>
-      <c r="Q290" s="5"/>
+      <c r="J290" s="5"/>
+      <c r="R290" s="5"/>
     </row>
     <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I291" s="5"/>
-      <c r="Q291" s="5"/>
+      <c r="J291" s="5"/>
+      <c r="R291" s="5"/>
     </row>
     <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I292" s="5"/>
-      <c r="Q292" s="5"/>
+      <c r="J292" s="5"/>
+      <c r="R292" s="5"/>
     </row>
     <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I293" s="5"/>
-      <c r="Q293" s="5"/>
+      <c r="J293" s="5"/>
+      <c r="R293" s="5"/>
     </row>
     <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I294" s="5"/>
-      <c r="Q294" s="5"/>
+      <c r="J294" s="5"/>
+      <c r="R294" s="5"/>
     </row>
     <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I295" s="5"/>
-      <c r="Q295" s="5"/>
+      <c r="J295" s="5"/>
+      <c r="R295" s="5"/>
     </row>
     <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I296" s="5"/>
-      <c r="Q296" s="5"/>
+      <c r="J296" s="5"/>
+      <c r="R296" s="5"/>
     </row>
     <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I297" s="5"/>
-      <c r="Q297" s="5"/>
+      <c r="J297" s="5"/>
+      <c r="R297" s="5"/>
     </row>
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I298" s="5"/>
-      <c r="Q298" s="5"/>
+      <c r="J298" s="5"/>
+      <c r="R298" s="5"/>
     </row>
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I299" s="5"/>
-      <c r="Q299" s="5"/>
+      <c r="J299" s="5"/>
+      <c r="R299" s="5"/>
     </row>
     <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I300" s="5"/>
-      <c r="Q300" s="5"/>
+      <c r="J300" s="5"/>
+      <c r="R300" s="5"/>
     </row>
     <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I301" s="5"/>
-      <c r="Q301" s="5"/>
+      <c r="J301" s="5"/>
+      <c r="R301" s="5"/>
     </row>
     <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I302" s="5"/>
-      <c r="Q302" s="5"/>
+      <c r="J302" s="5"/>
+      <c r="R302" s="5"/>
     </row>
     <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I303" s="5"/>
-      <c r="Q303" s="5"/>
+      <c r="J303" s="5"/>
+      <c r="R303" s="5"/>
     </row>
     <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I304" s="5"/>
-      <c r="Q304" s="5"/>
+      <c r="J304" s="5"/>
+      <c r="R304" s="5"/>
     </row>
     <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I305" s="5"/>
-      <c r="Q305" s="5"/>
+      <c r="J305" s="5"/>
+      <c r="R305" s="5"/>
     </row>
     <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I306" s="5"/>
-      <c r="Q306" s="5"/>
+      <c r="J306" s="5"/>
+      <c r="R306" s="5"/>
     </row>
     <row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I307" s="5"/>
-      <c r="Q307" s="5"/>
+      <c r="J307" s="5"/>
+      <c r="R307" s="5"/>
     </row>
     <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I308" s="5"/>
-      <c r="Q308" s="5"/>
+      <c r="J308" s="5"/>
+      <c r="R308" s="5"/>
     </row>
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I309" s="5"/>
-      <c r="Q309" s="5"/>
+      <c r="J309" s="5"/>
+      <c r="R309" s="5"/>
     </row>
     <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I310" s="5"/>
-      <c r="Q310" s="5"/>
+      <c r="J310" s="5"/>
+      <c r="R310" s="5"/>
     </row>
     <row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I311" s="5"/>
-      <c r="Q311" s="5"/>
+      <c r="J311" s="5"/>
+      <c r="R311" s="5"/>
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I312" s="5"/>
-      <c r="Q312" s="5"/>
+      <c r="J312" s="5"/>
+      <c r="R312" s="5"/>
     </row>
     <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I313" s="5"/>
-      <c r="Q313" s="5"/>
+      <c r="J313" s="5"/>
+      <c r="R313" s="5"/>
     </row>
     <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I314" s="5"/>
-      <c r="Q314" s="5"/>
+      <c r="J314" s="5"/>
+      <c r="R314" s="5"/>
     </row>
     <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I315" s="5"/>
-      <c r="Q315" s="5"/>
+      <c r="J315" s="5"/>
+      <c r="R315" s="5"/>
     </row>
     <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I316" s="5"/>
-      <c r="Q316" s="5"/>
+      <c r="J316" s="5"/>
+      <c r="R316" s="5"/>
     </row>
     <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I317" s="5"/>
-      <c r="Q317" s="5"/>
+      <c r="J317" s="5"/>
+      <c r="R317" s="5"/>
     </row>
     <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I318" s="5"/>
-      <c r="Q318" s="5"/>
+      <c r="J318" s="5"/>
+      <c r="R318" s="5"/>
     </row>
     <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I319" s="5"/>
-      <c r="Q319" s="5"/>
+      <c r="J319" s="5"/>
+      <c r="R319" s="5"/>
     </row>
     <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I320" s="5"/>
-      <c r="Q320" s="5"/>
+      <c r="J320" s="5"/>
+      <c r="R320" s="5"/>
     </row>
     <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I321" s="5"/>
-      <c r="Q321" s="5"/>
+      <c r="J321" s="5"/>
+      <c r="R321" s="5"/>
     </row>
     <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I322" s="5"/>
-      <c r="Q322" s="5"/>
+      <c r="J322" s="5"/>
+      <c r="R322" s="5"/>
     </row>
     <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I323" s="5"/>
-      <c r="Q323" s="5"/>
+      <c r="J323" s="5"/>
+      <c r="R323" s="5"/>
     </row>
     <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I324" s="5"/>
-      <c r="Q324" s="5"/>
+      <c r="J324" s="5"/>
+      <c r="R324" s="5"/>
     </row>
     <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I325" s="5"/>
-      <c r="Q325" s="5"/>
+      <c r="J325" s="5"/>
+      <c r="R325" s="5"/>
     </row>
     <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I326" s="5"/>
-      <c r="Q326" s="5"/>
+      <c r="J326" s="5"/>
+      <c r="R326" s="5"/>
     </row>
     <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I327" s="5"/>
-      <c r="Q327" s="5"/>
+      <c r="J327" s="5"/>
+      <c r="R327" s="5"/>
     </row>
     <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I328" s="5"/>
-      <c r="Q328" s="5"/>
+      <c r="J328" s="5"/>
+      <c r="R328" s="5"/>
     </row>
     <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I329" s="5"/>
-      <c r="Q329" s="5"/>
+      <c r="J329" s="5"/>
+      <c r="R329" s="5"/>
     </row>
     <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I330" s="5"/>
-      <c r="Q330" s="5"/>
+      <c r="J330" s="5"/>
+      <c r="R330" s="5"/>
     </row>
     <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I331" s="5"/>
-      <c r="Q331" s="5"/>
+      <c r="J331" s="5"/>
+      <c r="R331" s="5"/>
     </row>
     <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I332" s="5"/>
-      <c r="Q332" s="5"/>
+      <c r="J332" s="5"/>
+      <c r="R332" s="5"/>
     </row>
     <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I333" s="5"/>
-      <c r="Q333" s="5"/>
+      <c r="J333" s="5"/>
+      <c r="R333" s="5"/>
     </row>
     <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I334" s="5"/>
-      <c r="Q334" s="5"/>
+      <c r="J334" s="5"/>
+      <c r="R334" s="5"/>
     </row>
     <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I335" s="5"/>
-      <c r="Q335" s="5"/>
+      <c r="J335" s="5"/>
+      <c r="R335" s="5"/>
     </row>
     <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I336" s="5"/>
-      <c r="Q336" s="5"/>
+      <c r="J336" s="5"/>
+      <c r="R336" s="5"/>
     </row>
     <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I337" s="5"/>
-      <c r="Q337" s="5"/>
+      <c r="J337" s="5"/>
+      <c r="R337" s="5"/>
     </row>
     <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I338" s="5"/>
-      <c r="Q338" s="5"/>
+      <c r="J338" s="5"/>
+      <c r="R338" s="5"/>
     </row>
     <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I339" s="5"/>
-      <c r="Q339" s="5"/>
+      <c r="J339" s="5"/>
+      <c r="R339" s="5"/>
     </row>
     <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I340" s="5"/>
-      <c r="Q340" s="5"/>
+      <c r="J340" s="5"/>
+      <c r="R340" s="5"/>
     </row>
     <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I341" s="5"/>
-      <c r="Q341" s="5"/>
+      <c r="J341" s="5"/>
+      <c r="R341" s="5"/>
     </row>
     <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I342" s="5"/>
-      <c r="Q342" s="5"/>
+      <c r="J342" s="5"/>
+      <c r="R342" s="5"/>
     </row>
     <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I343" s="5"/>
-      <c r="Q343" s="5"/>
+      <c r="J343" s="5"/>
+      <c r="R343" s="5"/>
     </row>
     <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I344" s="5"/>
-      <c r="Q344" s="5"/>
+      <c r="J344" s="5"/>
+      <c r="R344" s="5"/>
     </row>
     <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I345" s="5"/>
-      <c r="Q345" s="5"/>
+      <c r="J345" s="5"/>
+      <c r="R345" s="5"/>
     </row>
     <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I346" s="5"/>
-      <c r="Q346" s="5"/>
+      <c r="J346" s="5"/>
+      <c r="R346" s="5"/>
     </row>
     <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I347" s="5"/>
-      <c r="Q347" s="5"/>
+      <c r="J347" s="5"/>
+      <c r="R347" s="5"/>
     </row>
     <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I348" s="5"/>
-      <c r="Q348" s="5"/>
+      <c r="J348" s="5"/>
+      <c r="R348" s="5"/>
     </row>
     <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I349" s="5"/>
-      <c r="Q349" s="5"/>
+      <c r="J349" s="5"/>
+      <c r="R349" s="5"/>
     </row>
     <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I350" s="5"/>
-      <c r="Q350" s="5"/>
+      <c r="J350" s="5"/>
+      <c r="R350" s="5"/>
     </row>
     <row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I351" s="5"/>
-      <c r="Q351" s="5"/>
+      <c r="J351" s="5"/>
+      <c r="R351" s="5"/>
     </row>
     <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I352" s="5"/>
-      <c r="Q352" s="5"/>
+      <c r="J352" s="5"/>
+      <c r="R352" s="5"/>
     </row>
     <row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I353" s="5"/>
-      <c r="Q353" s="5"/>
+      <c r="J353" s="5"/>
+      <c r="R353" s="5"/>
     </row>
     <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I354" s="5"/>
-      <c r="Q354" s="5"/>
+      <c r="J354" s="5"/>
+      <c r="R354" s="5"/>
     </row>
     <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I355" s="5"/>
-      <c r="Q355" s="5"/>
+      <c r="J355" s="5"/>
+      <c r="R355" s="5"/>
     </row>
     <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I356" s="5"/>
-      <c r="Q356" s="5"/>
-    </row>
-    <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I357" s="5"/>
-      <c r="Q357" s="5"/>
-    </row>
-    <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I358" s="5"/>
-      <c r="Q358" s="5"/>
-    </row>
-    <row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I359" s="5"/>
-      <c r="Q359" s="5"/>
-    </row>
-    <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I360" s="5"/>
-      <c r="Q360" s="5"/>
-    </row>
-    <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I361" s="5"/>
-      <c r="Q361" s="5"/>
-    </row>
-    <row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I362" s="5"/>
-      <c r="Q362" s="5"/>
-    </row>
-    <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I363" s="5"/>
-      <c r="Q363" s="5"/>
-    </row>
-    <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I364" s="5"/>
-      <c r="Q364" s="5"/>
-    </row>
-    <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I365" s="5"/>
-      <c r="Q365" s="5"/>
-    </row>
-    <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I366" s="5"/>
-      <c r="Q366" s="5"/>
-    </row>
-    <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I367" s="5"/>
-      <c r="Q367" s="5"/>
-    </row>
-    <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I368" s="5"/>
-      <c r="Q368" s="5"/>
-    </row>
-    <row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I369" s="5"/>
-      <c r="Q369" s="5"/>
-    </row>
-    <row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I370" s="5"/>
-      <c r="Q370" s="5"/>
-    </row>
-    <row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I371" s="5"/>
-      <c r="Q371" s="5"/>
-    </row>
+      <c r="J356" s="5"/>
+      <c r="R356" s="5"/>
+    </row>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:R369"/>
+  <autoFilter ref="B1:S354"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3082,58 +3169,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="Q1" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="R1" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3141,47 +3228,47 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" s="10"/>
       <c r="E2" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G2" s="12" t="n">
         <v>37125</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N2" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
       <c r="Q2" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R2" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3189,47 +3276,47 @@
         <v>1</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G3" s="12" t="n">
         <v>40777</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N3" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3237,47 +3324,47 @@
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G4" s="12" t="n">
         <v>33472</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N4" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
       <c r="Q4" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3285,47 +3372,47 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G5" s="12" t="n">
         <v>36760</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
       <c r="Q5" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>